<commit_message>
data: update 9 sources
</commit_message>
<xml_diff>
--- a/xlsx/Marnat.xlsx
+++ b/xlsx/Marnat.xlsx
@@ -49,7 +49,7 @@
     <t>Key</t>
   </si>
   <si>
-    <t>Part</t>
+    <t>Workpart</t>
   </si>
   <si>
     <t>Instrumentation</t>
@@ -100,7 +100,27 @@
     <t>Sérénade grotesque</t>
   </si>
   <si>
-    <t>Très rude (f♯)</t>
+    <r>
+      <t>Très rude (f</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♯</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)</t>
+    </r>
   </si>
   <si>
     <t>Solo Piano</t>
@@ -109,7 +129,27 @@
     <t>Un grand sommeil noir: Un grand sommeil noir</t>
   </si>
   <si>
-    <t>Lent et sourd mais jamais très marqué (c♯)</t>
+    <r>
+      <t>Lent et sourd mais jamais très marqué (c</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♯</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)</t>
+    </r>
   </si>
   <si>
     <t>Low Voice, Piano</t>
@@ -124,7 +164,27 @@
     <t>F-sharp minor</t>
   </si>
   <si>
-    <t>Maestoso (f♯)</t>
+    <r>
+      <t>Maestoso (f</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♯</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)</t>
+    </r>
   </si>
   <si>
     <t>arrangement for orchestra, Ravel, 1929 (Piccolo, 2 Flutes, 2 Oboes, English Horn, 2 Clarinets, Bass Clarinet, 2 Bassoon, Contrebassoon, 4 Horns, 3 Trumpets, 2 Trombones, Tuba, 2 Timpani, Harp, 2 Violins, Viola, Cello, Double Bass)</t>
@@ -133,14 +193,54 @@
     <t>Habanera</t>
   </si>
   <si>
-    <t>En demi-teinte et d'un rythme las (f♯)</t>
+    <r>
+      <t>En demi-teinte et d'un rythme las (f</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♯</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)</t>
+    </r>
   </si>
   <si>
     <t>2 Pianos</t>
   </si>
   <si>
-    <t>Sites auriculaires, ♯ 1
-transcription pour orchestre: 3è partie de la Rhapsodie espagnole ,1907 (voir ♯ 54 ci-dessous)</t>
+    <r>
+      <t xml:space="preserve">Sites auriculaires, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>#</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>1
+transcription pour orchestre: 3è partie de la Rhapsodie espagnole ,1907 (voir #54 ci-dessous)</t>
+    </r>
   </si>
   <si>
     <t>Sainte: À la fenêtre recélant</t>
@@ -164,7 +264,27 @@
     <t>C-sharp minor</t>
   </si>
   <si>
-    <t>Très léger et d'un rythme précis (c♯)</t>
+    <r>
+      <t>Très léger et d'un rythme précis (c</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♯</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)</t>
+    </r>
   </si>
   <si>
     <t>Voice, Harsichord/Piano</t>
@@ -238,7 +358,27 @@
     <t>Chanson du rouet: O mon cher rouet</t>
   </si>
   <si>
-    <t>Très lent (f♯)</t>
+    <r>
+      <t>Très lent (f</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♯</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)</t>
+    </r>
   </si>
   <si>
     <t>Texte: Leconte de Lisle</t>
@@ -256,10 +396,30 @@
     <t>3 Flutes, 3 Oboes, 2 Clarinets, 3 Bassoons, Sarrusophone, 4 Horns, 4 Trumpets, 3 Trombones, Tuba, Timpani, Percussion, Celesta, 2 Harps, 2 Violins, Viola, Cello, Double Bass</t>
   </si>
   <si>
-    <t>Inspiré de Milles et une nuits, traduction de Mardrus
+    <r>
+      <t xml:space="preserve">Inspiré de Milles et une nuits, traduction de Mardrus
 version originale pour piano quatre mains
 deux transcriptions pour orchestre «similaires mais non identiques»
-[aucun rapport avec Schéhérazade, ♯ 41 ci-dessous]</t>
+[aucun rapport avec Schéhérazade, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♯</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> 41 ci-dessous]</t>
+    </r>
   </si>
   <si>
     <t>1898-1899</t>
@@ -268,8 +428,28 @@
     <t>Olympia</t>
   </si>
   <si>
-    <t>Inspiré de l'Homme au sable d'Hoffman
-[esquisses détruites sauf une "symphonie horlogère" qui constitue le début de l'Heure espagnole ♯ 52 ci-dessous]</t>
+    <r>
+      <t xml:space="preserve">Inspiré de l'Homme au sable d'Hoffman
+[esquisses détruites sauf une "symphonie horlogère" qui constitue le début de l'Heure espagnole </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♯</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> 52 ci-dessous]</t>
+    </r>
   </si>
   <si>
     <t>Pavane pour une infante défunte</t>
@@ -295,7 +475,27 @@
     <t>D'Anne qui me jecta de la neige: Anne par jeu me jecta de la neige</t>
   </si>
   <si>
-    <t>Très lent (g♯)</t>
+    <r>
+      <t>Très lent (g</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♯</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)</t>
+    </r>
   </si>
   <si>
     <t>Texte: Clément Marot: Épigramme I, #11</t>
@@ -389,10 +589,30 @@
     <t>Quatuor</t>
   </si>
   <si>
-    <t>1. Allegro moderato (F)
+    <r>
+      <t>1. Allegro moderato (F)
 2. Assez vif, très rythmé (A)
-3. Très lent (G♭)
+3. Très lent (G</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♭</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)
 4. Vif et agité (F)</t>
+    </r>
   </si>
   <si>
     <t>Strings</t>
@@ -417,9 +637,29 @@
     <t>Manteau de fleurs: Toutes les fleurs de mon jardin sont roses</t>
   </si>
   <si>
-    <t>Texte: Paul Gravollet
+    <r>
+      <t xml:space="preserve">Texte: Paul Gravollet
 arrangement pour voix et orchestre, Ravel, sans date
-♯ 19 du recueil collectif intitulé Frissons: mélodies sur des textes de Paul Gravollet</t>
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♯</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> 19 du recueil collectif intitulé Frissons: mélodies sur des textes de Paul Gravollet</t>
+    </r>
   </si>
   <si>
     <t>1903-1905</t>
@@ -428,14 +668,126 @@
     <t>Sonatine</t>
   </si>
   <si>
-    <t>1. Modéré (f♯)
-2. Mouvement de menuet (D♭)
-3. Animé (f♯)</t>
-  </si>
-  <si>
-    <t>1. Asie: Asie, Asie. Très lent (e♭)(Piccolo, 2 Flutes, 2 Oboes, English Horn, 2 Clarinets, 2 Bassoon, 4 Horns, 2 Trumpets, 3 Trombones, Tuba, Timpani, Triangle, Basque Drum, Side Drum, Cymbal, Bass Drum, Tam-tam, jeu de Timbres, 2 Harps, 2 Violins, Viola, Cello, Double Bass) 
-2. La Flute enchantée: L'ombre est douce et ton maître dort. Très lent (b♭)(2 Flutes, 2 Oboes, English Horn, 2 Clarinets, 2 Bassoon, 4 Horns, Triangle, Harp, 2 Violins, Viola, Cello, Double Bass) 
-3. L'indifférent: Tes yeux sont doux comme ceux d'une fille. Lent (c♯)(2 Flutes, 2 Oboes, English Horn, 2 Clarinets, 2 Bassoon, 2 Horns, Harp, 2 Violins, Viola, Cello, Double Bass)</t>
+    <r>
+      <t>1. Modéré (f</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♯</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)
+2. Mouvement de menuet (D</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♭</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)
+3. Animé (f</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♯</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>1. Asie: Asie, Asie. Très lent (e</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♭</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)(Piccolo, 2 Flutes, 2 Oboes, English Horn, 2 Clarinets, 2 Bassoon, 4 Horns, 2 Trumpets, 3 Trombones, Tuba, Timpani, Triangle, Basque Drum, Side Drum, Cymbal, Bass Drum, Tam-tam, jeu de Timbres, 2 Harps, 2 Violins, Viola, Cello, Double Bass) 
+2. La Flute enchantée: L'ombre est douce et ton maître dort. Très lent (b</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♭</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)(2 Flutes, 2 Oboes, English Horn, 2 Clarinets, 2 Bassoon, 4 Horns, Triangle, Harp, 2 Violins, Viola, Cello, Double Bass) 
+3. L'indifférent: Tes yeux sont doux comme ceux d'une fille. Lent (c</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♯</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)(2 Flutes, 2 Oboes, English Horn, 2 Clarinets, 2 Bassoon, 2 Horns, Harp, 2 Violins, Viola, Cello, Double Bass)</t>
+    </r>
   </si>
   <si>
     <t>S/T, 3 Flutes, 3 Oboes, 2 Clarinets, 2 Bassoons, 4 Horns, 2 Trumpets, 3 Trombones, Tuba, 2 Timpani, jeu de Timbres, Tam-tam, Percussions, carillon, Celesta, 3 Harps, 2 Violins, Viola, Cello, Double Bass</t>
@@ -453,11 +805,85 @@
     <t>Miroirs</t>
   </si>
   <si>
-    <t>1. Noctuelles. Très léger (D♭)
-2. Oiseaux tristes. Très lent (e♭)
-3. Une barque sur l'océan. D'un rythme souple (f♯)
+    <r>
+      <t>1. Noctuelles. Très léger (D</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♭</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)
+2. Oiseaux tristes. Très lent (e</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♭</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)
+3. Une barque sur l'océan. D'un rythme souple (f</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♯</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)
 4. Alborada del gracioso. Assez vif (d)
-5. La vallée des cloches. Très lent (c♯)</t>
+5. La vallée des cloches. Très lent (c</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♯</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)</t>
+    </r>
   </si>
   <si>
     <t>1904/05, original: Piano
@@ -477,8 +903,46 @@
     <t>Introduction et allegro</t>
   </si>
   <si>
-    <t>1. Introduction. Très lent (G♭)
-2. Allegro (G♭)</t>
+    <r>
+      <t>1. Introduction. Très lent (G</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♭</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)
+2. Allegro (G</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♭</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)</t>
+    </r>
   </si>
   <si>
     <t>Harp, Flute, Clarinet, 2 Violins, Viola et Cello</t>
@@ -494,7 +958,27 @@
     <t>Les grands vents d'outre-mer: Les grands vents venus d'outre-mer</t>
   </si>
   <si>
-    <t>Modéré, très agité (E♭)</t>
+    <r>
+      <t>Modéré, très agité (E</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♭</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)</t>
+    </r>
   </si>
   <si>
     <t>Texte: Henri de Régnier</t>
@@ -516,11 +1000,31 @@
     <t>Histoires naturelles</t>
   </si>
   <si>
-    <t>1. Le paon: Il va surement se marier aujourd'hui Sans hâte et noblement (F)
+    <r>
+      <t>1. Le paon: Il va surement se marier aujourd'hui Sans hâte et noblement (F)
 2. Le grillon: C'est l'heure où, las d'errer Placide (a)
 3. Le cygne: Il glisse sur le bassin Lent (B)
-4. Le martin-pêcheur: Ça n'a pas mordu, ce soir On ne peut plus lent (F♯)
+4. Le martin-pêcheur: Ça n'a pas mordu, ce soir On ne peut plus lent (F</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♯</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)
 5. La pintade: C'est la bossue de ma cour Assez vite (E)</t>
+    </r>
   </si>
   <si>
     <t>Medium Voice, Piano</t>
@@ -568,7 +1072,27 @@
     <t>Sur l'herbe: L'abbé divague. Et toi, marquis</t>
   </si>
   <si>
-    <t>Modéré (c♯)</t>
+    <r>
+      <t>Modéré (c</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♯</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)</t>
+    </r>
   </si>
   <si>
     <t>Rhapsodie espagnole, pour orchestre</t>
@@ -625,9 +1149,47 @@
     <t>Gaspard de la nuit</t>
   </si>
   <si>
-    <t>1. Ondine Lent (C♯)
-2. Le gibet Très lent (e♭)
+    <r>
+      <t>1. Ondine Lent (C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♯</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)
+2. Le gibet Très lent (e</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♭</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)
 3. Scarbo Modéré (B)</t>
+    </r>
   </si>
   <si>
     <t>after Aloysius Bertrand</t>
@@ -829,14 +1391,34 @@
     <t>Valses nobles et sentimentales</t>
   </si>
   <si>
-    <t>1. Modéré - très franc (G)
+    <r>
+      <t>1. Modéré - très franc (G)
 2. Assez lent - avec une expression intense (g)
 3. Modéré (e)
-4. Assez animé (A♭)
+4. Assez animé (A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♭</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)
 5. Presque lent - dans un sentiment intime (E)
 6. Vif (C)
 7. Moins vif (C / A)
 8. Épilogue. Lent (G)</t>
+    </r>
   </si>
   <si>
     <t>Piano
@@ -852,13 +1434,69 @@
     <t>Ma mère l'oye (II), musique de ballet</t>
   </si>
   <si>
-    <t>1. Prélude
+    <r>
+      <t>1. Prélude
 2. Danse du rouet et scène
 3. Pavane de la belle au bois dormant(2 Flutes, Oboes, English Horn, 2 Clarinets, Bassoon, Horn, Harp, cordes) Lent (a)
 4. Entretiens de la belle et de la bête(2 Flutes, Oboes, English Horn, 2 Clarinets, 2 Bassoon, 2 Horns, Timpani, Cymbal, Triangle, jeu de Timbres, Celesta, Harp, cordes) Mouvement de valse. Modéré (F)
-5. Petit poucet(2 Flutes, Oboes, English Horn, 2 Clarinets, 2 Bassoon, 2 Horns, cordes) Très modéré (E♭)
-6. Laideronnette, impératrice des pagodes(Piccolo, Flute, Oboes, English Horn, 2 Clarinets, 2 Bassoon, 2 Horns, Timpani, Cymbal, Tam-tam, Xylophone, jeu de Timbres, Celesta, Harp, cordes) Mouvement de marche (F♯)
-7. Apothéose. Le jardin féerique(2 Flutes, 2 Oboes, 2 Clarinets, Bassoon, contre♭asson, 2 Horns, Triangle, Cymbal, Bass Drum, Harp, cordes) Lent et grave (C)</t>
+5. Petit poucet(2 Flutes, Oboes, English Horn, 2 Clarinets, 2 Bassoon, 2 Horns, cordes) Très modéré (E</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♭</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)
+6. Laideronnette, impératrice des pagodes(Piccolo, Flute, Oboes, English Horn, 2 Clarinets, 2 Bassoon, 2 Horns, Timpani, Cymbal, Tam-tam, Xylophone, jeu de Timbres, Celesta, Harp, cordes) Mouvement de marche (F</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♯</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)
+7. Apothéose. Le jardin féerique(2 Flutes, 2 Oboes, 2 Clarinets, Bassoon, contre</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♭</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>asson, 2 Horns, Triangle, Cymbal, Bass Drum, Harp, cordes) Lent et grave (C)</t>
+    </r>
   </si>
   <si>
     <t>Piccolo, Flute, Oboes, English Horn, 2 Clarinets, Bassoon, Contrebassoon, 2 Horns, 2 Timpani, Triangle, Cymbal, Bass Drum, Tam-tam, Xylophone, Celesta, Harp, 2 Violins, Viola, Cello, Double Bass</t>
@@ -950,10 +1588,30 @@
     <t>Trio</t>
   </si>
   <si>
-    <t>1. Modéré (a)
+    <r>
+      <t>1. Modéré (a)
 2. Pantoum. Assez vite (a)
-3. Passacaille. Très large (f♯)
+3. Passacaille. Très large (f</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♯</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)
 4. Final. Animé (A)</t>
+    </r>
   </si>
   <si>
     <t>Piano, Violin, Cello</t>
@@ -1101,9 +1759,29 @@
     <t>1923-1927</t>
   </si>
   <si>
-    <t>1. Allegretto (G)
-2. Blues. Moderato (A♯)
+    <r>
+      <t>1. Allegretto (G)
+2. Blues. Moderato (A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♯</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)
 3. Perpetuum mobile. Allegro (G)</t>
+    </r>
   </si>
   <si>
     <r>
@@ -1208,9 +1886,47 @@
     <t>Don Quichotte à Dulcinée</t>
   </si>
   <si>
-    <t>1. Chanson romanesque: Si vous me disiez que la terre Moderato (b♭/B♭)
+    <r>
+      <t>1. Chanson romanesque: Si vous me disiez que la terre Moderato (b</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♭</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>/B</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>♭</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)
 2. Chanson épique: Bon Saint Michel qui me donnez loisir Molto moderato (F)
 3. Chanson à boire: Foin du bâtard, illustre Dame Allegro (C)</t>
+    </r>
   </si>
   <si>
     <t>Bar, 2 Flutes, 3 Oboes, 2 Clarinets, 2 Bassoons, Horn, Trumpet, Castanets, vibraphone, Harp, 2 Violins, Viola, Cello, Double Bass</t>
@@ -1874,7 +2590,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1893,12 +2609,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1906,34 +2622,16 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -2461,31 +3159,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G92"/>
-  <sheetFormatPr defaultColWidth="8.61261261261261" defaultRowHeight="25" customHeight="1" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="8.61261261261261" defaultRowHeight="30" customHeight="1" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="10.4954954954955" style="3" customWidth="1"/>
-    <col min="2" max="2" width="11.3603603603604" style="3" customWidth="1"/>
-    <col min="3" max="3" width="65.5585585585586" style="4" customWidth="1"/>
+    <col min="1" max="2" width="14.4414414414414" style="3" customWidth="1"/>
+    <col min="3" max="3" width="23.7027027027027" style="4" customWidth="1"/>
     <col min="4" max="4" width="14.5855855855856" style="3" customWidth="1"/>
-    <col min="5" max="5" width="34.972972972973" style="5" customWidth="1"/>
-    <col min="6" max="7" width="34.972972972973" style="6" customWidth="1"/>
+    <col min="5" max="7" width="23.7027027027027" style="5" customWidth="1"/>
     <col min="8" max="16384" width="8.61261261261261" style="2"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" customHeight="1" spans="1:7">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="7" t="s">
@@ -2506,11 +3202,11 @@
         <v>7</v>
       </c>
       <c r="D2" s="8"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="11" t="s">
+      <c r="E2" s="9"/>
+      <c r="F2" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="10" t="s">
         <v>9</v>
       </c>
     </row>
@@ -2521,15 +3217,15 @@
       <c r="B3" s="8">
         <v>1888</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D3" s="8"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="11" t="s">
+      <c r="E3" s="9"/>
+      <c r="F3" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G3" s="11" t="s">
+      <c r="G3" s="10" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2540,15 +3236,15 @@
       <c r="B4" s="8">
         <v>1888</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D4" s="8"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="11" t="s">
+      <c r="E4" s="9"/>
+      <c r="F4" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="11" t="s">
+      <c r="G4" s="10" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2559,82 +3255,82 @@
       <c r="B5" s="8">
         <v>1893</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="F5" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="G5" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="6" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A6" s="8">
         <v>5</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="9" t="s">
         <v>20</v>
       </c>
       <c r="D6" s="8"/>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="G6" s="13"/>
-    </row>
-    <row r="7" s="2" customFormat="1" ht="15.4" spans="1:7">
+      <c r="G6" s="10"/>
+    </row>
+    <row r="7" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A7" s="8">
         <v>6</v>
       </c>
       <c r="B7" s="8">
         <v>1895</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="9" t="s">
         <v>23</v>
       </c>
       <c r="D7" s="8"/>
-      <c r="E7" s="11" t="s">
+      <c r="E7" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F7" s="11" t="s">
+      <c r="F7" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="G7" s="10" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="8" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="8" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A8" s="8">
         <v>7</v>
       </c>
       <c r="B8" s="8">
         <v>1895</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="D8" s="12" t="s">
+      <c r="D8" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="G8" s="10" t="s">
         <v>30</v>
       </c>
     </row>
@@ -2645,17 +3341,17 @@
       <c r="B9" s="8">
         <v>1895</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="9" t="s">
         <v>31</v>
       </c>
       <c r="D9" s="8"/>
-      <c r="E9" s="11" t="s">
+      <c r="E9" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="F9" s="11" t="s">
+      <c r="F9" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="G9" s="10" t="s">
         <v>34</v>
       </c>
     </row>
@@ -2666,19 +3362,19 @@
       <c r="B10" s="8">
         <v>1896</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="E10" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="F10" s="11" t="s">
+      <c r="F10" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="G10" s="11" t="s">
+      <c r="G10" s="10" t="s">
         <v>39</v>
       </c>
     </row>
@@ -2689,19 +3385,19 @@
       <c r="B11" s="8">
         <v>1896</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="12" t="s">
+      <c r="D11" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="E11" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="F11" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="G11" s="11" t="s">
+      <c r="G11" s="10" t="s">
         <v>44</v>
       </c>
     </row>
@@ -2712,17 +3408,17 @@
       <c r="B12" s="8">
         <v>1896</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="9" t="s">
         <v>45</v>
       </c>
       <c r="D12" s="8"/>
-      <c r="E12" s="11" t="s">
+      <c r="E12" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="F12" s="11" t="s">
+      <c r="F12" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G12" s="11" t="s">
+      <c r="G12" s="10" t="s">
         <v>47</v>
       </c>
     </row>
@@ -2733,634 +3429,634 @@
       <c r="B13" s="8">
         <v>1897</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="11" t="s">
         <v>48</v>
       </c>
       <c r="D13" s="8"/>
-      <c r="E13" s="11" t="s">
+      <c r="E13" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="F13" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="G13" s="11" t="s">
+      <c r="G13" s="10" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="14" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="14" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A14" s="8">
         <v>13</v>
       </c>
       <c r="B14" s="8">
         <v>1897</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="D14" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="E14" s="11" t="s">
+      <c r="E14" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="F14" s="11" t="s">
+      <c r="F14" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="G14" s="11" t="s">
+      <c r="G14" s="10" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="15" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="15" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A15" s="8">
         <v>14</v>
       </c>
       <c r="B15" s="8">
         <v>1898</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="D15" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="E15" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="F15" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G15" s="13"/>
-    </row>
-    <row r="16" s="2" customFormat="1" ht="15.4" spans="1:7">
+      <c r="G15" s="10"/>
+    </row>
+    <row r="16" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A16" s="8">
         <v>15</v>
       </c>
       <c r="B16" s="8">
         <v>1898</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="C16" s="9" t="s">
         <v>59</v>
       </c>
       <c r="D16" s="8"/>
-      <c r="E16" s="11" t="s">
+      <c r="E16" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="F16" s="11" t="s">
+      <c r="F16" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G16" s="11" t="s">
+      <c r="G16" s="10" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="17" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="17" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A17" s="8">
         <v>16</v>
       </c>
       <c r="B17" s="8">
         <v>1898</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="9" t="s">
         <v>62</v>
       </c>
       <c r="D17" s="8"/>
-      <c r="E17" s="11" t="s">
+      <c r="E17" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="F17" s="11" t="s">
+      <c r="F17" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G17" s="11" t="s">
+      <c r="G17" s="10" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="18" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="18" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A18" s="8">
         <v>17</v>
       </c>
       <c r="B18" s="8">
         <v>1898</v>
       </c>
-      <c r="C18" s="11" t="s">
+      <c r="C18" s="9" t="s">
         <v>64</v>
       </c>
       <c r="D18" s="8"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="15" t="s">
+      <c r="E18" s="9"/>
+      <c r="F18" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="G18" s="11" t="s">
+      <c r="G18" s="10" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="19" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="19" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A19" s="8">
         <v>18</v>
       </c>
-      <c r="B19" s="12" t="s">
+      <c r="B19" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="C19" s="11" t="s">
+      <c r="C19" s="9" t="s">
         <v>68</v>
       </c>
       <c r="D19" s="8"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="11" t="s">
+      <c r="E19" s="9"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="20" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="20" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A20" s="8">
         <v>19</v>
       </c>
       <c r="B20" s="8">
         <v>1899</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="D20" s="12" t="s">
+      <c r="D20" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="E20" s="11" t="s">
+      <c r="E20" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="F20" s="11" t="s">
+      <c r="F20" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G20" s="11" t="s">
+      <c r="G20" s="10" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="21" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="21" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A21" s="8">
         <v>20</v>
       </c>
       <c r="B21" s="8">
         <v>1899</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="9" t="s">
         <v>74</v>
       </c>
       <c r="D21" s="8"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="11" t="s">
+      <c r="E21" s="9"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="22" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="22" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A22" s="8">
         <v>21</v>
       </c>
       <c r="B22" s="8">
         <v>1899</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="9" t="s">
         <v>76</v>
       </c>
       <c r="D22" s="8"/>
-      <c r="E22" s="11" t="s">
+      <c r="E22" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="F22" s="11" t="s">
+      <c r="F22" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G22" s="11" t="s">
+      <c r="G22" s="10" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="23" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="23" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A23" s="8">
         <v>22</v>
       </c>
       <c r="B23" s="8">
         <v>1900</v>
       </c>
-      <c r="C23" s="11" t="s">
+      <c r="C23" s="9" t="s">
         <v>79</v>
       </c>
       <c r="D23" s="8"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="11" t="s">
+      <c r="E23" s="9"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="24" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="24" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A24" s="8">
         <v>23</v>
       </c>
       <c r="B24" s="8">
         <v>1900</v>
       </c>
-      <c r="C24" s="11" t="s">
+      <c r="C24" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="D24" s="12" t="s">
+      <c r="D24" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="E24" s="10"/>
-      <c r="F24" s="11" t="s">
+      <c r="E24" s="9"/>
+      <c r="F24" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G24" s="11" t="s">
+      <c r="G24" s="10" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="25" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="25" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A25" s="8">
         <v>24</v>
       </c>
       <c r="B25" s="8">
         <v>1900</v>
       </c>
-      <c r="C25" s="11" t="s">
+      <c r="C25" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="D25" s="12" t="s">
+      <c r="D25" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="E25" s="10"/>
-      <c r="F25" s="11" t="s">
+      <c r="E25" s="9"/>
+      <c r="F25" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G25" s="13"/>
-    </row>
-    <row r="26" s="2" customFormat="1" ht="15.4" spans="1:7">
+      <c r="G25" s="10"/>
+    </row>
+    <row r="26" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A26" s="8">
         <v>25</v>
       </c>
       <c r="B26" s="8">
         <v>1900</v>
       </c>
-      <c r="C26" s="11" t="s">
+      <c r="C26" s="9" t="s">
         <v>84</v>
       </c>
       <c r="D26" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="E26" s="10"/>
-      <c r="F26" s="11" t="s">
+      <c r="E26" s="9"/>
+      <c r="F26" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="G26" s="11" t="s">
+      <c r="G26" s="10" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="27" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="27" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A27" s="8">
         <v>26</v>
       </c>
       <c r="B27" s="8">
         <v>1900</v>
       </c>
-      <c r="C27" s="11" t="s">
+      <c r="C27" s="9" t="s">
         <v>87</v>
       </c>
       <c r="D27" s="8"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="11" t="s">
+      <c r="E27" s="9"/>
+      <c r="F27" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G27" s="11" t="s">
+      <c r="G27" s="10" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="28" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="28" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A28" s="8">
         <v>27</v>
       </c>
       <c r="B28" s="8">
         <v>1900</v>
       </c>
-      <c r="C28" s="11" t="s">
+      <c r="C28" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="D28" s="12" t="s">
+      <c r="D28" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="E28" s="10"/>
-      <c r="F28" s="11" t="s">
+      <c r="E28" s="9"/>
+      <c r="F28" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G28" s="11" t="s">
+      <c r="G28" s="10" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="29" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="29" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A29" s="8">
         <v>28</v>
       </c>
       <c r="B29" s="8">
         <v>1901</v>
       </c>
-      <c r="C29" s="11" t="s">
+      <c r="C29" s="9" t="s">
         <v>89</v>
       </c>
       <c r="D29" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="E29" s="10"/>
-      <c r="F29" s="11" t="s">
+      <c r="E29" s="9"/>
+      <c r="F29" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="G29" s="11" t="s">
+      <c r="G29" s="10" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="30" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="30" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A30" s="8">
         <v>29</v>
       </c>
       <c r="B30" s="8">
         <v>1901</v>
       </c>
-      <c r="C30" s="11" t="s">
+      <c r="C30" s="9" t="s">
         <v>92</v>
       </c>
       <c r="D30" s="8"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="11" t="s">
+      <c r="E30" s="9"/>
+      <c r="F30" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="G30" s="11" t="s">
+      <c r="G30" s="10" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="31" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="31" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A31" s="8">
         <v>30</v>
       </c>
       <c r="B31" s="8">
         <v>1901</v>
       </c>
-      <c r="C31" s="11" t="s">
+      <c r="C31" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="D31" s="12" t="s">
+      <c r="D31" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="E31" s="11" t="s">
+      <c r="E31" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="F31" s="11" t="s">
+      <c r="F31" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G31" s="13"/>
-    </row>
-    <row r="32" s="2" customFormat="1" ht="15.4" spans="1:7">
+      <c r="G31" s="10"/>
+    </row>
+    <row r="32" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A32" s="8">
         <v>31</v>
       </c>
       <c r="B32" s="8">
         <v>1902</v>
       </c>
-      <c r="C32" s="11" t="s">
+      <c r="C32" s="9" t="s">
         <v>98</v>
       </c>
       <c r="D32" s="8"/>
-      <c r="E32" s="10"/>
-      <c r="F32" s="13"/>
-      <c r="G32" s="11" t="s">
+      <c r="E32" s="9"/>
+      <c r="F32" s="10"/>
+      <c r="G32" s="10" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="33" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="33" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A33" s="8">
         <v>32</v>
       </c>
       <c r="B33" s="8">
         <v>1902</v>
       </c>
-      <c r="C33" s="11" t="s">
+      <c r="C33" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="D33" s="12" t="s">
+      <c r="D33" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="E33" s="10"/>
-      <c r="F33" s="11" t="s">
+      <c r="E33" s="9"/>
+      <c r="F33" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G33" s="11" t="s">
+      <c r="G33" s="10" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="34" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="34" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A34" s="8">
         <v>33</v>
       </c>
       <c r="B34" s="8">
         <v>1902</v>
       </c>
-      <c r="C34" s="11" t="s">
+      <c r="C34" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="D34" s="12" t="s">
+      <c r="D34" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="E34" s="10"/>
-      <c r="F34" s="11" t="s">
+      <c r="E34" s="9"/>
+      <c r="F34" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="G34" s="11" t="s">
+      <c r="G34" s="10" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="35" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="35" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A35" s="8">
         <v>34</v>
       </c>
       <c r="B35" s="8">
         <v>1902</v>
       </c>
-      <c r="C35" s="11" t="s">
+      <c r="C35" s="9" t="s">
         <v>102</v>
       </c>
       <c r="D35" s="8"/>
-      <c r="E35" s="10"/>
-      <c r="F35" s="13"/>
-      <c r="G35" s="11" t="s">
+      <c r="E35" s="9"/>
+      <c r="F35" s="10"/>
+      <c r="G35" s="10" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="36" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="36" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A36" s="8">
         <v>35</v>
       </c>
-      <c r="B36" s="12" t="s">
+      <c r="B36" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="C36" s="11" t="s">
+      <c r="C36" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="D36" s="12" t="s">
+      <c r="D36" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="E36" s="11" t="s">
+      <c r="E36" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="F36" s="11" t="s">
+      <c r="F36" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="G36" s="13"/>
-    </row>
-    <row r="37" s="2" customFormat="1" ht="15.4" spans="1:7">
+      <c r="G36" s="10"/>
+    </row>
+    <row r="37" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A37" s="8">
         <v>36</v>
       </c>
       <c r="B37" s="8">
         <v>1903</v>
       </c>
-      <c r="C37" s="11" t="s">
+      <c r="C37" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="D37" s="12" t="s">
+      <c r="D37" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="E37" s="10"/>
-      <c r="F37" s="11" t="s">
+      <c r="E37" s="9"/>
+      <c r="F37" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G37" s="11" t="s">
+      <c r="G37" s="10" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="38" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="38" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A38" s="8">
         <v>37</v>
       </c>
       <c r="B38" s="8">
         <v>1903</v>
       </c>
-      <c r="C38" s="11" t="s">
+      <c r="C38" s="9" t="s">
         <v>109</v>
       </c>
       <c r="D38" s="8"/>
-      <c r="E38" s="10"/>
-      <c r="F38" s="11" t="s">
+      <c r="E38" s="9"/>
+      <c r="F38" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="G38" s="11" t="s">
+      <c r="G38" s="10" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="39" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="39" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A39" s="8">
         <v>38</v>
       </c>
       <c r="B39" s="8">
         <v>1903</v>
       </c>
-      <c r="C39" s="11" t="s">
+      <c r="C39" s="9" t="s">
         <v>111</v>
       </c>
       <c r="D39" s="8"/>
-      <c r="E39" s="10"/>
-      <c r="F39" s="11" t="s">
+      <c r="E39" s="9"/>
+      <c r="F39" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="G39" s="11" t="s">
+      <c r="G39" s="10" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="40" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="40" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A40" s="8">
         <v>39</v>
       </c>
       <c r="B40" s="8">
         <v>1903</v>
       </c>
-      <c r="C40" s="11" t="s">
+      <c r="C40" s="9" t="s">
         <v>113</v>
       </c>
       <c r="D40" s="8"/>
-      <c r="E40" s="10"/>
-      <c r="F40" s="11" t="s">
+      <c r="E40" s="9"/>
+      <c r="F40" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G40" s="11" t="s">
+      <c r="G40" s="10" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="41" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="41" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A41" s="8">
         <v>40</v>
       </c>
-      <c r="B41" s="12" t="s">
+      <c r="B41" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="C41" s="11" t="s">
+      <c r="C41" s="9" t="s">
         <v>116</v>
       </c>
       <c r="D41" s="8"/>
-      <c r="E41" s="11" t="s">
+      <c r="E41" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="F41" s="11" t="s">
+      <c r="F41" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G41" s="13"/>
-    </row>
-    <row r="42" s="2" customFormat="1" ht="15.4" spans="1:7">
+      <c r="G41" s="10"/>
+    </row>
+    <row r="42" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A42" s="8">
         <v>41</v>
       </c>
       <c r="B42" s="8">
         <v>1903</v>
       </c>
-      <c r="C42" s="11" t="s">
+      <c r="C42" s="9" t="s">
         <v>64</v>
       </c>
       <c r="D42" s="8"/>
-      <c r="E42" s="11" t="s">
+      <c r="E42" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="F42" s="15" t="s">
+      <c r="F42" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="G42" s="11" t="s">
+      <c r="G42" s="10" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="43" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="43" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A43" s="8">
         <v>42</v>
       </c>
       <c r="B43" s="8">
         <v>1904</v>
       </c>
-      <c r="C43" s="11" t="s">
+      <c r="C43" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="D43" s="12" t="s">
+      <c r="D43" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="E43" s="10"/>
-      <c r="F43" s="11" t="s">
+      <c r="E43" s="9"/>
+      <c r="F43" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G43" s="13"/>
-    </row>
-    <row r="44" s="2" customFormat="1" ht="15.4" spans="1:7">
+      <c r="G43" s="10"/>
+    </row>
+    <row r="44" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A44" s="8">
         <v>43</v>
       </c>
-      <c r="B44" s="12" t="s">
+      <c r="B44" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="C44" s="11" t="s">
+      <c r="C44" s="9" t="s">
         <v>123</v>
       </c>
       <c r="D44" s="8"/>
-      <c r="E44" s="11" t="s">
+      <c r="E44" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="F44" s="15" t="s">
+      <c r="F44" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="G44" s="13"/>
+      <c r="G44" s="10"/>
     </row>
     <row r="45" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A45" s="8">
@@ -3369,59 +4065,59 @@
       <c r="B45" s="8">
         <v>1905</v>
       </c>
-      <c r="C45" s="11" t="s">
+      <c r="C45" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="D45" s="12" t="s">
+      <c r="D45" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="E45" s="10"/>
-      <c r="F45" s="11" t="s">
+      <c r="E45" s="9"/>
+      <c r="F45" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G45" s="11" t="s">
+      <c r="G45" s="10" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="46" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="46" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A46" s="8">
         <v>45</v>
       </c>
       <c r="B46" s="8">
         <v>1905</v>
       </c>
-      <c r="C46" s="11" t="s">
+      <c r="C46" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="D46" s="12" t="s">
+      <c r="D46" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="E46" s="10"/>
-      <c r="F46" s="11" t="s">
+      <c r="E46" s="9"/>
+      <c r="F46" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="G46" s="11" t="s">
+      <c r="G46" s="10" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="47" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="47" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A47" s="8">
         <v>46</v>
       </c>
       <c r="B47" s="8">
         <v>1905</v>
       </c>
-      <c r="C47" s="11" t="s">
+      <c r="C47" s="9" t="s">
         <v>129</v>
       </c>
       <c r="D47" s="8"/>
-      <c r="E47" s="11" t="s">
+      <c r="E47" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="F47" s="11" t="s">
+      <c r="F47" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="G47" s="13"/>
+      <c r="G47" s="10"/>
     </row>
     <row r="48" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A48" s="8">
@@ -3430,362 +4126,362 @@
       <c r="B48" s="8">
         <v>1905</v>
       </c>
-      <c r="C48" s="11" t="s">
+      <c r="C48" s="9" t="s">
         <v>132</v>
       </c>
       <c r="D48" s="8"/>
-      <c r="E48" s="10"/>
-      <c r="F48" s="11" t="s">
+      <c r="E48" s="9"/>
+      <c r="F48" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G48" s="11" t="s">
+      <c r="G48" s="10" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="49" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="49" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A49" s="8">
         <v>48</v>
       </c>
       <c r="B49" s="8">
         <v>1906</v>
       </c>
-      <c r="C49" s="11" t="s">
+      <c r="C49" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="D49" s="12" t="s">
+      <c r="D49" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="E49" s="11" t="s">
+      <c r="E49" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="F49" s="11" t="s">
+      <c r="F49" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G49" s="11" t="s">
+      <c r="G49" s="10" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="50" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="50" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A50" s="8">
         <v>49</v>
       </c>
-      <c r="B50" s="12" t="s">
+      <c r="B50" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="C50" s="11" t="s">
+      <c r="C50" s="9" t="s">
         <v>138</v>
       </c>
       <c r="D50" s="8"/>
-      <c r="E50" s="10"/>
-      <c r="F50" s="11" t="s">
+      <c r="E50" s="9"/>
+      <c r="F50" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="G50" s="11" t="s">
+      <c r="G50" s="10" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="51" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="51" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A51" s="8">
         <v>50</v>
       </c>
       <c r="B51" s="8">
         <v>1906</v>
       </c>
-      <c r="C51" s="11" t="s">
+      <c r="C51" s="9" t="s">
         <v>141</v>
       </c>
       <c r="D51" s="8"/>
-      <c r="E51" s="11" t="s">
+      <c r="E51" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="F51" s="11" t="s">
+      <c r="F51" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="G51" s="11" t="s">
+      <c r="G51" s="10" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="52" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="52" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A52" s="8">
         <v>51</v>
       </c>
       <c r="B52" s="8">
         <v>1907</v>
       </c>
-      <c r="C52" s="11" t="s">
+      <c r="C52" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="D52" s="12" t="s">
+      <c r="D52" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="E52" s="11" t="s">
+      <c r="E52" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="F52" s="11" t="s">
+      <c r="F52" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="G52" s="13"/>
-    </row>
-    <row r="53" s="2" customFormat="1" ht="154.3" spans="1:7">
+      <c r="G52" s="10"/>
+    </row>
+    <row r="53" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A53" s="8">
         <v>52</v>
       </c>
       <c r="B53" s="8">
         <v>1907</v>
       </c>
-      <c r="C53" s="11" t="s">
+      <c r="C53" s="9" t="s">
         <v>147</v>
       </c>
       <c r="D53" s="8"/>
-      <c r="E53" s="10"/>
-      <c r="F53" s="16" t="s">
+      <c r="E53" s="9"/>
+      <c r="F53" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="G53" s="16" t="s">
+      <c r="G53" s="10" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="54" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="54" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A54" s="8">
         <v>53</v>
       </c>
       <c r="B54" s="8">
         <v>1907</v>
       </c>
-      <c r="C54" s="11" t="s">
+      <c r="C54" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="D54" s="12" t="s">
+      <c r="D54" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="E54" s="11" t="s">
+      <c r="E54" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="F54" s="11" t="s">
+      <c r="F54" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G54" s="11" t="s">
+      <c r="G54" s="10" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="55" s="2" customFormat="1" ht="138.85" spans="1:7">
+    <row r="55" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A55" s="8">
         <v>54</v>
       </c>
       <c r="B55" s="8">
         <v>1907</v>
       </c>
-      <c r="C55" s="11" t="s">
+      <c r="C55" s="9" t="s">
         <v>152</v>
       </c>
       <c r="D55" s="8"/>
-      <c r="E55" s="11" t="s">
+      <c r="E55" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="F55" s="17" t="s">
+      <c r="F55" s="10" t="s">
         <v>154</v>
       </c>
-      <c r="G55" s="11"/>
-    </row>
-    <row r="56" s="2" customFormat="1" ht="15.4" spans="1:7">
+      <c r="G55" s="10"/>
+    </row>
+    <row r="56" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A56" s="8">
         <v>55</v>
       </c>
       <c r="B56" s="8">
         <v>1908</v>
       </c>
-      <c r="C56" s="11" t="s">
+      <c r="C56" s="9" t="s">
         <v>155</v>
       </c>
       <c r="D56" s="8"/>
-      <c r="E56" s="11" t="s">
+      <c r="E56" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="F56" s="11" t="s">
+      <c r="F56" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G56" s="11" t="s">
+      <c r="G56" s="10" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="57" s="2" customFormat="1" ht="46.3" spans="1:7">
+    <row r="57" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A57" s="8">
         <v>56</v>
       </c>
       <c r="B57" s="8">
         <v>1908</v>
       </c>
-      <c r="C57" s="11" t="s">
+      <c r="C57" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="D57" s="12" t="s">
+      <c r="D57" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="E57" s="11" t="s">
+      <c r="E57" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="F57" s="11" t="s">
+      <c r="F57" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="G57" s="16" t="s">
+      <c r="G57" s="10" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="58" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="58" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A58" s="8">
         <v>57</v>
       </c>
-      <c r="B58" s="12" t="s">
+      <c r="B58" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="C58" s="11" t="s">
+      <c r="C58" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="D58" s="12" t="s">
+      <c r="D58" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="E58" s="11"/>
-      <c r="F58" s="15" t="s">
+      <c r="E58" s="9"/>
+      <c r="F58" s="10" t="s">
         <v>165</v>
       </c>
-      <c r="G58" s="11" t="s">
+      <c r="G58" s="10" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="59" s="2" customFormat="1" ht="15.45" spans="1:7">
-      <c r="A59" s="12" t="s">
+    <row r="59" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="A59" s="8" t="s">
         <v>167</v>
       </c>
       <c r="B59" s="8">
         <v>1911</v>
       </c>
-      <c r="C59" s="11" t="s">
+      <c r="C59" s="9" t="s">
         <v>164</v>
       </c>
       <c r="D59" s="8"/>
-      <c r="E59" s="11" t="s">
+      <c r="E59" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="F59" s="18"/>
-      <c r="G59" s="19" t="s">
+      <c r="F59" s="12"/>
+      <c r="G59" s="13" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="60" s="2" customFormat="1" ht="15.4" spans="1:7">
-      <c r="A60" s="12" t="s">
+    <row r="60" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="A60" s="8" t="s">
         <v>170</v>
       </c>
       <c r="B60" s="8">
         <v>1913</v>
       </c>
-      <c r="C60" s="11" t="s">
+      <c r="C60" s="9" t="s">
         <v>164</v>
       </c>
       <c r="D60" s="8"/>
-      <c r="E60" s="11" t="s">
+      <c r="E60" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="F60" s="18"/>
-      <c r="G60" s="19" t="s">
+      <c r="F60" s="12"/>
+      <c r="G60" s="13" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="61" s="2" customFormat="1" ht="15.4" spans="1:7">
-      <c r="A61" s="12" t="s">
+    <row r="61" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="A61" s="8" t="s">
         <v>173</v>
       </c>
       <c r="B61" s="8">
         <v>1913</v>
       </c>
-      <c r="C61" s="11" t="s">
+      <c r="C61" s="9" t="s">
         <v>174</v>
       </c>
       <c r="D61" s="8"/>
-      <c r="E61" s="11" t="s">
+      <c r="E61" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="F61" s="11" t="s">
+      <c r="F61" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G61" s="13"/>
-    </row>
-    <row r="62" s="2" customFormat="1" ht="15.4" spans="1:7">
+      <c r="G61" s="10"/>
+    </row>
+    <row r="62" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A62" s="8">
         <v>58</v>
       </c>
       <c r="B62" s="8">
         <v>1909</v>
       </c>
-      <c r="C62" s="11" t="s">
+      <c r="C62" s="9" t="s">
         <v>176</v>
       </c>
       <c r="D62" s="8"/>
-      <c r="E62" s="10"/>
-      <c r="F62" s="11" t="s">
+      <c r="E62" s="9"/>
+      <c r="F62" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G62" s="19" t="s">
+      <c r="G62" s="13" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="63" s="2" customFormat="1" ht="46.3" spans="1:7">
+    <row r="63" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A63" s="8">
         <v>59</v>
       </c>
-      <c r="B63" s="12" t="s">
+      <c r="B63" s="8" t="s">
         <v>178</v>
       </c>
-      <c r="C63" s="11" t="s">
+      <c r="C63" s="9" t="s">
         <v>179</v>
       </c>
       <c r="D63" s="8"/>
-      <c r="E63" s="10"/>
-      <c r="F63" s="11" t="s">
+      <c r="E63" s="9"/>
+      <c r="F63" s="10" t="s">
         <v>180</v>
       </c>
-      <c r="G63" s="16" t="s">
+      <c r="G63" s="10" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="64" s="2" customFormat="1" ht="61.7" spans="1:7">
+    <row r="64" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A64" s="8">
         <v>60</v>
       </c>
-      <c r="B64" s="12" t="s">
+      <c r="B64" s="8" t="s">
         <v>182</v>
       </c>
-      <c r="C64" s="11" t="s">
+      <c r="C64" s="9" t="s">
         <v>183</v>
       </c>
       <c r="D64" s="8"/>
-      <c r="E64" s="11" t="s">
+      <c r="E64" s="9" t="s">
         <v>184</v>
       </c>
-      <c r="F64" s="11" t="s">
+      <c r="F64" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="G64" s="16" t="s">
+      <c r="G64" s="10" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="65" s="2" customFormat="1" ht="108" spans="1:7">
+    <row r="65" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A65" s="8">
         <v>61</v>
       </c>
       <c r="B65" s="8">
         <v>1911</v>
       </c>
-      <c r="C65" s="11" t="s">
+      <c r="C65" s="9" t="s">
         <v>186</v>
       </c>
       <c r="D65" s="8"/>
-      <c r="E65" s="11" t="s">
+      <c r="E65" s="9" t="s">
         <v>187</v>
       </c>
-      <c r="F65" s="16" t="s">
+      <c r="F65" s="10" t="s">
         <v>188</v>
       </c>
-      <c r="G65" s="16" t="s">
+      <c r="G65" s="10" t="s">
         <v>189</v>
       </c>
     </row>
@@ -3793,538 +4489,538 @@
       <c r="A66" s="8">
         <v>62</v>
       </c>
-      <c r="B66" s="12" t="s">
+      <c r="B66" s="8" t="s">
         <v>190</v>
       </c>
-      <c r="C66" s="11" t="s">
+      <c r="C66" s="9" t="s">
         <v>191</v>
       </c>
       <c r="D66" s="8"/>
-      <c r="E66" s="11" t="s">
+      <c r="E66" s="9" t="s">
         <v>192</v>
       </c>
-      <c r="F66" s="11" t="s">
+      <c r="F66" s="10" t="s">
         <v>193</v>
       </c>
-      <c r="G66" s="11" t="s">
+      <c r="G66" s="10" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="67" s="2" customFormat="1" ht="15.45" spans="1:7">
+    <row r="67" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A67" s="8">
         <v>63</v>
       </c>
-      <c r="B67" s="12" t="s">
+      <c r="B67" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="C67" s="11" t="s">
+      <c r="C67" s="9" t="s">
         <v>196</v>
       </c>
       <c r="D67" s="8"/>
-      <c r="E67" s="11" t="s">
+      <c r="E67" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="F67" s="11" t="s">
+      <c r="F67" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G67" s="11" t="s">
+      <c r="G67" s="10" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="68" s="2" customFormat="1" ht="61.7" spans="1:7">
+    <row r="68" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A68" s="8">
         <v>64</v>
       </c>
       <c r="B68" s="8">
         <v>1913</v>
       </c>
-      <c r="C68" s="11" t="s">
+      <c r="C68" s="9" t="s">
         <v>199</v>
       </c>
       <c r="D68" s="8"/>
-      <c r="E68" s="11" t="s">
+      <c r="E68" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="F68" s="16" t="s">
+      <c r="F68" s="10" t="s">
         <v>201</v>
       </c>
-      <c r="G68" s="16" t="s">
+      <c r="G68" s="10" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="69" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="69" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A69" s="8">
         <v>65</v>
       </c>
       <c r="B69" s="8">
         <v>1913</v>
       </c>
-      <c r="C69" s="11" t="s">
+      <c r="C69" s="9" t="s">
         <v>202</v>
       </c>
       <c r="D69" s="8"/>
-      <c r="E69" s="10"/>
-      <c r="F69" s="11" t="s">
+      <c r="E69" s="9"/>
+      <c r="F69" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G69" s="13"/>
+      <c r="G69" s="10"/>
     </row>
     <row r="70" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A70" s="8">
         <v>66</v>
       </c>
-      <c r="B70" s="12" t="s">
+      <c r="B70" s="8" t="s">
         <v>203</v>
       </c>
-      <c r="C70" s="11" t="s">
+      <c r="C70" s="9" t="s">
         <v>204</v>
       </c>
       <c r="D70" s="8"/>
-      <c r="E70" s="10"/>
-      <c r="F70" s="11" t="s">
+      <c r="E70" s="9"/>
+      <c r="F70" s="10" t="s">
         <v>205</v>
       </c>
-      <c r="G70" s="11" t="s">
+      <c r="G70" s="10" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="71" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="71" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A71" s="8">
         <v>67</v>
       </c>
       <c r="B71" s="8">
         <v>1914</v>
       </c>
-      <c r="C71" s="14" t="s">
+      <c r="C71" s="11" t="s">
         <v>207</v>
       </c>
-      <c r="D71" s="12" t="s">
+      <c r="D71" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="E71" s="11" t="s">
+      <c r="E71" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="F71" s="11" t="s">
+      <c r="F71" s="10" t="s">
         <v>209</v>
       </c>
-      <c r="G71" s="13"/>
-    </row>
-    <row r="72" s="2" customFormat="1" ht="15.4" spans="1:7">
+      <c r="G71" s="10"/>
+    </row>
+    <row r="72" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A72" s="8">
         <v>68</v>
       </c>
-      <c r="B72" s="12" t="s">
+      <c r="B72" s="8" t="s">
         <v>210</v>
       </c>
-      <c r="C72" s="11" t="s">
+      <c r="C72" s="9" t="s">
         <v>211</v>
       </c>
       <c r="D72" s="8"/>
-      <c r="E72" s="11" t="s">
+      <c r="E72" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="F72" s="11" t="s">
+      <c r="F72" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G72" s="13"/>
-    </row>
-    <row r="73" s="2" customFormat="1" ht="15.4" spans="1:7">
-      <c r="A73" s="12" t="s">
+      <c r="G72" s="10"/>
+    </row>
+    <row r="73" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="A73" s="8" t="s">
         <v>213</v>
       </c>
       <c r="B73" s="8">
         <v>1919</v>
       </c>
-      <c r="C73" s="11" t="s">
+      <c r="C73" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="D73" s="12" t="s">
+      <c r="D73" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="E73" s="11" t="s">
+      <c r="E73" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="F73" s="15" t="s">
+      <c r="F73" s="10" t="s">
         <v>215</v>
       </c>
-      <c r="G73" s="13"/>
-    </row>
-    <row r="74" s="2" customFormat="1" ht="30.85" spans="1:7">
+      <c r="G73" s="10"/>
+    </row>
+    <row r="74" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A74" s="8">
         <v>69</v>
       </c>
-      <c r="B74" s="12" t="s">
+      <c r="B74" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="C74" s="11" t="s">
+      <c r="C74" s="9" t="s">
         <v>217</v>
       </c>
       <c r="D74" s="8"/>
-      <c r="E74" s="11" t="s">
+      <c r="E74" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="F74" s="16" t="s">
+      <c r="F74" s="10" t="s">
         <v>219</v>
       </c>
-      <c r="G74" s="16" t="s">
+      <c r="G74" s="10" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="75" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="75" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A75" s="8">
         <v>70</v>
       </c>
       <c r="B75" s="8">
         <v>1918</v>
       </c>
-      <c r="C75" s="11" t="s">
+      <c r="C75" s="9" t="s">
         <v>221</v>
       </c>
       <c r="D75" s="8"/>
-      <c r="E75" s="11" t="s">
+      <c r="E75" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="F75" s="11" t="s">
+      <c r="F75" s="10" t="s">
         <v>223</v>
       </c>
-      <c r="G75" s="11" t="s">
+      <c r="G75" s="10" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="76" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="76" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A76" s="8">
         <v>71</v>
       </c>
-      <c r="B76" s="12" t="s">
+      <c r="B76" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="C76" s="11" t="s">
+      <c r="C76" s="9" t="s">
         <v>226</v>
       </c>
       <c r="D76" s="8"/>
-      <c r="E76" s="10"/>
-      <c r="F76" s="15" t="s">
+      <c r="E76" s="9"/>
+      <c r="F76" s="10" t="s">
         <v>227</v>
       </c>
-      <c r="G76" s="11" t="s">
+      <c r="G76" s="10" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="77" s="2" customFormat="1" ht="138.85" spans="1:7">
+    <row r="77" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A77" s="8">
         <v>72</v>
       </c>
-      <c r="B77" s="12" t="s">
+      <c r="B77" s="8" t="s">
         <v>229</v>
       </c>
-      <c r="C77" s="11" t="s">
+      <c r="C77" s="9" t="s">
         <v>230</v>
       </c>
-      <c r="D77" s="12" t="s">
+      <c r="D77" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="E77" s="11" t="s">
+      <c r="E77" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="F77" s="17" t="s">
+      <c r="F77" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="G77" s="11"/>
-    </row>
-    <row r="78" s="2" customFormat="1" ht="15.4" spans="1:7">
+      <c r="G77" s="10"/>
+    </row>
+    <row r="78" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A78" s="8">
         <v>73</v>
       </c>
-      <c r="B78" s="12" t="s">
+      <c r="B78" s="8" t="s">
         <v>233</v>
       </c>
-      <c r="C78" s="14" t="s">
+      <c r="C78" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="D78" s="12" t="s">
+      <c r="D78" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="E78" s="11" t="s">
+      <c r="E78" s="9" t="s">
         <v>234</v>
       </c>
-      <c r="F78" s="11" t="s">
+      <c r="F78" s="10" t="s">
         <v>235</v>
       </c>
-      <c r="G78" s="11" t="s">
+      <c r="G78" s="10" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="79" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="79" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A79" s="8">
         <v>74</v>
       </c>
       <c r="B79" s="8">
         <v>1922</v>
       </c>
-      <c r="C79" s="11" t="s">
+      <c r="C79" s="9" t="s">
         <v>237</v>
       </c>
-      <c r="D79" s="12" t="s">
+      <c r="D79" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="E79" s="11" t="s">
+      <c r="E79" s="9" t="s">
         <v>238</v>
       </c>
-      <c r="F79" s="11" t="s">
+      <c r="F79" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="G79" s="13"/>
-    </row>
-    <row r="80" s="2" customFormat="1" ht="77.15" spans="1:7">
+      <c r="G79" s="10"/>
+    </row>
+    <row r="80" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A80" s="8">
         <v>75</v>
       </c>
-      <c r="B80" s="12" t="s">
+      <c r="B80" s="8" t="s">
         <v>239</v>
       </c>
-      <c r="C80" s="11" t="s">
+      <c r="C80" s="9" t="s">
         <v>240</v>
       </c>
       <c r="D80" s="8"/>
-      <c r="E80" s="10"/>
-      <c r="F80" s="16" t="s">
+      <c r="E80" s="9"/>
+      <c r="F80" s="10" t="s">
         <v>241</v>
       </c>
-      <c r="G80" s="16" t="s">
+      <c r="G80" s="10" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="81" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="81" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A81" s="8">
         <v>76</v>
       </c>
-      <c r="B81" s="12" t="s">
+      <c r="B81" s="8" t="s">
         <v>243</v>
       </c>
-      <c r="C81" s="11" t="s">
+      <c r="C81" s="9" t="s">
         <v>244</v>
       </c>
-      <c r="D81" s="12" t="s">
+      <c r="D81" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="E81" s="11" t="s">
+      <c r="E81" s="9" t="s">
         <v>245</v>
       </c>
-      <c r="F81" s="11" t="s">
+      <c r="F81" s="10" t="s">
         <v>246</v>
       </c>
-      <c r="G81" s="13"/>
-    </row>
-    <row r="82" s="2" customFormat="1" ht="15.45" spans="1:7">
+      <c r="G81" s="10"/>
+    </row>
+    <row r="82" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A82" s="8">
         <v>77</v>
       </c>
-      <c r="B82" s="12" t="s">
+      <c r="B82" s="8" t="s">
         <v>247</v>
       </c>
-      <c r="C82" s="14" t="s">
+      <c r="C82" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="D82" s="12" t="s">
+      <c r="D82" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="E82" s="11" t="s">
+      <c r="E82" s="9" t="s">
         <v>248</v>
       </c>
-      <c r="F82" s="11" t="s">
+      <c r="F82" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="G82" s="11" t="s">
+      <c r="G82" s="10" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="83" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="83" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A83" s="8">
         <v>78</v>
       </c>
-      <c r="B83" s="12" t="s">
+      <c r="B83" s="8" t="s">
         <v>250</v>
       </c>
-      <c r="C83" s="11" t="s">
+      <c r="C83" s="9" t="s">
         <v>251</v>
       </c>
       <c r="D83" s="8"/>
-      <c r="E83" s="11" t="s">
+      <c r="E83" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="F83" s="11" t="s">
+      <c r="F83" s="10" t="s">
         <v>253</v>
       </c>
-      <c r="G83" s="11" t="s">
+      <c r="G83" s="10" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="84" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="84" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A84" s="8">
         <v>79</v>
       </c>
       <c r="B84" s="8">
         <v>1927</v>
       </c>
-      <c r="C84" s="11" t="s">
+      <c r="C84" s="9" t="s">
         <v>255</v>
       </c>
       <c r="D84" s="8"/>
-      <c r="E84" s="10"/>
-      <c r="F84" s="11" t="s">
+      <c r="E84" s="9"/>
+      <c r="F84" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G84" s="11" t="s">
+      <c r="G84" s="10" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="85" s="2" customFormat="1" ht="61.7" spans="1:7">
+    <row r="85" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A85" s="8">
         <v>80</v>
       </c>
       <c r="B85" s="8">
         <v>1927</v>
       </c>
-      <c r="C85" s="11" t="s">
+      <c r="C85" s="9" t="s">
         <v>257</v>
       </c>
       <c r="D85" s="8"/>
-      <c r="E85" s="10"/>
-      <c r="F85" s="16" t="s">
+      <c r="E85" s="9"/>
+      <c r="F85" s="10" t="s">
         <v>258</v>
       </c>
-      <c r="G85" s="11"/>
-    </row>
-    <row r="86" s="2" customFormat="1" ht="15.4" spans="1:7">
+      <c r="G85" s="10"/>
+    </row>
+    <row r="86" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A86" s="8">
         <v>81</v>
       </c>
       <c r="B86" s="8">
         <v>1928</v>
       </c>
-      <c r="C86" s="11" t="s">
+      <c r="C86" s="9" t="s">
         <v>259</v>
       </c>
-      <c r="D86" s="12" t="s">
+      <c r="D86" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="E86" s="11" t="s">
+      <c r="E86" s="9" t="s">
         <v>260</v>
       </c>
-      <c r="F86" s="15" t="s">
+      <c r="F86" s="10" t="s">
         <v>261</v>
       </c>
-      <c r="G86" s="11" t="s">
+      <c r="G86" s="10" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="87" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="87" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A87" s="8">
         <v>82</v>
       </c>
-      <c r="B87" s="12" t="s">
+      <c r="B87" s="8" t="s">
         <v>263</v>
       </c>
-      <c r="C87" s="11" t="s">
+      <c r="C87" s="9" t="s">
         <v>264</v>
       </c>
-      <c r="D87" s="12" t="s">
+      <c r="D87" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="E87" s="11" t="s">
+      <c r="E87" s="9" t="s">
         <v>265</v>
       </c>
-      <c r="F87" s="15" t="s">
+      <c r="F87" s="10" t="s">
         <v>266</v>
       </c>
-      <c r="G87" s="11" t="s">
+      <c r="G87" s="10" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="88" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="88" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A88" s="8">
         <v>83</v>
       </c>
-      <c r="B88" s="12" t="s">
+      <c r="B88" s="8" t="s">
         <v>268</v>
       </c>
-      <c r="C88" s="11" t="s">
+      <c r="C88" s="9" t="s">
         <v>264</v>
       </c>
-      <c r="D88" s="12" t="s">
+      <c r="D88" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="E88" s="11" t="s">
+      <c r="E88" s="9" t="s">
         <v>269</v>
       </c>
-      <c r="F88" s="11" t="s">
+      <c r="F88" s="10" t="s">
         <v>270</v>
       </c>
-      <c r="G88" s="11" t="s">
+      <c r="G88" s="10" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="89" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="89" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A89" s="8">
         <v>84</v>
       </c>
-      <c r="B89" s="12" t="s">
+      <c r="B89" s="8" t="s">
         <v>272</v>
       </c>
-      <c r="C89" s="11" t="s">
+      <c r="C89" s="9" t="s">
         <v>273</v>
       </c>
       <c r="D89" s="8"/>
-      <c r="E89" s="11" t="s">
+      <c r="E89" s="9" t="s">
         <v>274</v>
       </c>
-      <c r="F89" s="15" t="s">
+      <c r="F89" s="10" t="s">
         <v>275</v>
       </c>
-      <c r="G89" s="11" t="s">
+      <c r="G89" s="10" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="90" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="90" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A90" s="8">
         <v>85</v>
       </c>
       <c r="B90" s="8">
         <v>1932</v>
       </c>
-      <c r="C90" s="11" t="s">
+      <c r="C90" s="9" t="s">
         <v>277</v>
       </c>
       <c r="D90" s="8"/>
-      <c r="E90" s="10"/>
-      <c r="F90" s="11" t="s">
+      <c r="E90" s="9"/>
+      <c r="F90" s="10" t="s">
         <v>278</v>
       </c>
-      <c r="G90" s="11" t="s">
+      <c r="G90" s="10" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="91" s="2" customFormat="1" ht="15.4" spans="1:7">
+    <row r="91" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A91" s="3"/>
       <c r="B91" s="3"/>
       <c r="C91" s="4"/>
       <c r="D91" s="3"/>
       <c r="E91" s="5"/>
-      <c r="F91" s="6"/>
-      <c r="G91" s="6"/>
-    </row>
-    <row r="92" s="2" customFormat="1" ht="15.4" spans="1:7">
+      <c r="F91" s="5"/>
+      <c r="G91" s="5"/>
+    </row>
+    <row r="92" s="2" customFormat="1" customHeight="1" spans="1:7">
       <c r="A92" s="3"/>
       <c r="B92" s="3"/>
       <c r="C92" s="4"/>
       <c r="D92" s="3"/>
       <c r="E92" s="5"/>
-      <c r="F92" s="6"/>
-      <c r="G92" s="6"/>
+      <c r="F92" s="5"/>
+      <c r="G92" s="5"/>
     </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:G92" etc:filterBottomFollowUsedRange="0">
-    <sortState ref="A2:G92">
+    <sortState ref="A1:G92">
       <sortCondition ref="A1"/>
     </sortState>
     <extLst/>

</xml_diff>

<commit_message>
added SORTing for Marnat
</commit_message>
<xml_diff>
--- a/xlsx/Marnat.xlsx
+++ b/xlsx/Marnat.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$92</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +35,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="367">
+  <si>
+    <t>SORT</t>
+  </si>
   <si>
     <t>Catalogue</t>
   </si>
@@ -58,6 +61,9 @@
     <t>Note</t>
   </si>
   <si>
+    <t>M. 1</t>
+  </si>
+  <si>
     <t>Mouvement de sonate</t>
   </si>
   <si>
@@ -67,18 +73,30 @@
     <t>Exercice pour les cours de Charles-René, [perdu]</t>
   </si>
   <si>
+    <t xml:space="preserve">M. </t>
+  </si>
+  <si>
+    <t>M. 2</t>
+  </si>
+  <si>
     <t>Variations sur un thème de Grieg</t>
   </si>
   <si>
     <t>Exercice pour les cours de Charles-René, "La mort d'Aase", extrait de la musique de scène pour le Peer Gynt d'Ibsen</t>
   </si>
   <si>
+    <t>M. 3</t>
+  </si>
+  <si>
     <t>Variations sur un thème de Schumann</t>
   </si>
   <si>
     <t>Exercice pour les cours de Charles-René, Choral "Freu dich, o meine Seele" de l'Album pour la jeunesse (Op. 68)</t>
   </si>
   <si>
+    <t>M. 4</t>
+  </si>
+  <si>
     <t>Ballade de la reine morte d'aimer: En Bohème était une reine</t>
   </si>
   <si>
@@ -94,6 +112,9 @@
     <t>Texte: Roland de Marès</t>
   </si>
   <si>
+    <t>M. 5</t>
+  </si>
+  <si>
     <t>1892-1893</t>
   </si>
   <si>
@@ -101,6 +122,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t>Très rude (f</t>
     </r>
     <r>
@@ -126,10 +153,19 @@
     <t>Solo Piano</t>
   </si>
   <si>
+    <t>M. 6</t>
+  </si>
+  <si>
     <t>Un grand sommeil noir: Un grand sommeil noir</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t>Lent et sourd mais jamais très marqué (c</t>
     </r>
     <r>
@@ -158,6 +194,9 @@
     <t>Texte: Paul Verlaine</t>
   </si>
   <si>
+    <t>M. 7</t>
+  </si>
+  <si>
     <t>Menuet antique</t>
   </si>
   <si>
@@ -165,6 +204,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t>Maestoso (f</t>
     </r>
     <r>
@@ -190,10 +235,19 @@
     <t>arrangement for orchestra, Ravel, 1929 (Piccolo, 2 Flutes, 2 Oboes, English Horn, 2 Clarinets, Bass Clarinet, 2 Bassoon, Contrebassoon, 4 Horns, 3 Trumpets, 2 Trombones, Tuba, 2 Timpani, Harp, 2 Violins, Viola, Cello, Double Bass)</t>
   </si>
   <si>
+    <t>M. 8</t>
+  </si>
+  <si>
     <t>Habanera</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t>En demi-teinte et d'un rythme las (f</t>
     </r>
     <r>
@@ -220,6 +274,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Sites auriculaires, </t>
     </r>
     <r>
@@ -243,6 +303,9 @@
     </r>
   </si>
   <si>
+    <t>M. 9</t>
+  </si>
+  <si>
     <t>Sainte: À la fenêtre recélant</t>
   </si>
   <si>
@@ -258,6 +321,9 @@
     <t>Texte: Stéphane Mallarmé</t>
   </si>
   <si>
+    <t>M. 10</t>
+  </si>
+  <si>
     <t>D'Anne jouant de l'espinette: Lorsque je voy en ordre la brunette</t>
   </si>
   <si>
@@ -265,6 +331,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t>Très léger et d'un rythme précis (c</t>
     </r>
     <r>
@@ -291,6 +363,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Texte:Clément Marot: Épigramme II, </t>
     </r>
     <r>
@@ -313,6 +391,9 @@
     </r>
   </si>
   <si>
+    <t>M. 11</t>
+  </si>
+  <si>
     <t>La parade</t>
   </si>
   <si>
@@ -322,6 +403,9 @@
     <t>Esquisse de ballet d'après un livret d'Antonine Meunier</t>
   </si>
   <si>
+    <t>M. 12</t>
+  </si>
+  <si>
     <t>Sonata</t>
   </si>
   <si>
@@ -334,6 +418,9 @@
     <t>Sonate #1</t>
   </si>
   <si>
+    <t>M. 13</t>
+  </si>
+  <si>
     <t>Entre cloches</t>
   </si>
   <si>
@@ -346,6 +433,9 @@
     <t>Sites auriculaires, #2</t>
   </si>
   <si>
+    <t>M. 14</t>
+  </si>
+  <si>
     <t>Valse</t>
   </si>
   <si>
@@ -355,10 +445,19 @@
     <t>Moderato (E)</t>
   </si>
   <si>
+    <t>M. 15</t>
+  </si>
+  <si>
     <t>Chanson du rouet: O mon cher rouet</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t>Très lent (f</t>
     </r>
     <r>
@@ -384,12 +483,18 @@
     <t>Texte: Leconte de Lisle</t>
   </si>
   <si>
+    <t>M. 16</t>
+  </si>
+  <si>
     <t>Si morne!: Se replier toujours, sur soi-même</t>
   </si>
   <si>
     <t>Texte:Émile Verhaeren</t>
   </si>
   <si>
+    <t>M. 17</t>
+  </si>
+  <si>
     <t>Schéhérazade</t>
   </si>
   <si>
@@ -397,6 +502,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Inspiré de Milles et une nuits, traduction de Mardrus
 version originale pour piano quatre mains
 deux transcriptions pour orchestre «similaires mais non identiques»
@@ -422,6 +533,9 @@
     </r>
   </si>
   <si>
+    <t>M. 18</t>
+  </si>
+  <si>
     <t>1898-1899</t>
   </si>
   <si>
@@ -429,6 +543,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Inspiré de l'Homme au sable d'Hoffman
 [esquisses détruites sauf une "symphonie horlogère" qui constitue le début de l'Heure espagnole </t>
     </r>
@@ -452,6 +572,9 @@
     </r>
   </si>
   <si>
+    <t>M. 19</t>
+  </si>
+  <si>
     <t>Pavane pour une infante défunte</t>
   </si>
   <si>
@@ -465,6 +588,9 @@
 (2 Flutes, Oboes, 2 Clarinets, 2 Bassoon, Horn, Harp, 2 Violins, Viola, Cello, Double Bass)</t>
   </si>
   <si>
+    <t>M. 20</t>
+  </si>
+  <si>
     <t>Fugue</t>
   </si>
   <si>
@@ -472,10 +598,19 @@
 [Lost]</t>
   </si>
   <si>
+    <t>M. 21</t>
+  </si>
+  <si>
     <t>D'Anne qui me jecta de la neige: Anne par jeu me jecta de la neige</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t>Très lent (g</t>
     </r>
     <r>
@@ -499,6 +634,9 @@
   </si>
   <si>
     <t>Texte: Clément Marot: Épigramme I, #11</t>
+  </si>
+  <si>
+    <t>M. 22</t>
   </si>
   <si>
     <t>Callerhoe</t>
@@ -508,13 +646,22 @@
 Pièce pour le concours d'essai au prix de Rome</t>
   </si>
   <si>
+    <t>M. 23</t>
+  </si>
+  <si>
     <t>Pièce de concours pour le prix de Rome</t>
   </si>
   <si>
+    <t>M. 24</t>
+  </si>
+  <si>
     <t>Fugue à quatre voix sur un thème de Reber</t>
   </si>
   <si>
     <t>F major</t>
+  </si>
+  <si>
+    <t>M. 25</t>
   </si>
   <si>
     <t>Les Bayadères</t>
@@ -527,6 +674,9 @@
 Pièce de concours pour le prix de Rome</t>
   </si>
   <si>
+    <t>M. 26</t>
+  </si>
+  <si>
     <t>Prélude et fugue</t>
   </si>
   <si>
@@ -534,6 +684,12 @@
 [perdu]</t>
   </si>
   <si>
+    <t>M. 27</t>
+  </si>
+  <si>
+    <t>M. 28</t>
+  </si>
+  <si>
     <t>Tout est lumière</t>
   </si>
   <si>
@@ -544,6 +700,9 @@
 Pièce de concours pour le prix de Rome</t>
   </si>
   <si>
+    <t>M. 29</t>
+  </si>
+  <si>
     <t>Myrrha</t>
   </si>
   <si>
@@ -554,6 +713,9 @@
 Pièce de concours pour le prix de Rome</t>
   </si>
   <si>
+    <t>M. 30</t>
+  </si>
+  <si>
     <t>Jeux d'eau</t>
   </si>
   <si>
@@ -561,6 +723,9 @@
   </si>
   <si>
     <t>Très doux (E)</t>
+  </si>
+  <si>
+    <t>M. 31</t>
   </si>
   <si>
     <t>Semiramis</t>
@@ -570,10 +735,19 @@
 [perdu]</t>
   </si>
   <si>
+    <t>M. 32</t>
+  </si>
+  <si>
     <t>E-flat major</t>
   </si>
   <si>
+    <t>M. 33</t>
+  </si>
+  <si>
     <t>La nuit</t>
+  </si>
+  <si>
+    <t>M. 34</t>
   </si>
   <si>
     <t>Alcyone</t>
@@ -583,6 +757,9 @@
 Pièce de concours pour le prix de Rome</t>
   </si>
   <si>
+    <t>M. 35</t>
+  </si>
+  <si>
     <t>1902-1903</t>
   </si>
   <si>
@@ -590,6 +767,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t>1. Allegro moderato (F)
 2. Assez vif, très rythmé (A)
 3. Très lent (G</t>
@@ -618,13 +801,22 @@
     <t>Strings</t>
   </si>
   <si>
+    <t>M. 36</t>
+  </si>
+  <si>
     <t>E minor</t>
   </si>
   <si>
+    <t>M. 37</t>
+  </si>
+  <si>
     <t>Matinée de Provence</t>
   </si>
   <si>
     <t>pièce chorale, en A, pour soprano et choeur mixte avec orchestre</t>
+  </si>
+  <si>
+    <t>M. 38</t>
   </si>
   <si>
     <t>Alyssa</t>
@@ -634,10 +826,19 @@
 Pièce de concours pour le prix de Rome</t>
   </si>
   <si>
+    <t>M. 39</t>
+  </si>
+  <si>
     <t>Manteau de fleurs: Toutes les fleurs de mon jardin sont roses</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Texte: Paul Gravollet
 arrangement pour voix et orchestre, Ravel, sans date
 </t>
@@ -662,6 +863,9 @@
     </r>
   </si>
   <si>
+    <t>M. 40</t>
+  </si>
+  <si>
     <t>1903-1905</t>
   </si>
   <si>
@@ -669,6 +873,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t>1. Modéré (f</t>
     </r>
     <r>
@@ -729,7 +939,16 @@
     </r>
   </si>
   <si>
-    <r>
+    <t>M. 41</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t>1. Asie: Asie, Asie. Très lent (e</t>
     </r>
     <r>
@@ -796,9 +1015,15 @@
     <t>Texte: Tristan Klingsor</t>
   </si>
   <si>
+    <t>M. 42</t>
+  </si>
+  <si>
     <t>Menuet</t>
   </si>
   <si>
+    <t>M. 43</t>
+  </si>
+  <si>
     <t>1904-1905</t>
   </si>
   <si>
@@ -806,6 +1031,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t>1. Noctuelles. Très léger (D</t>
     </r>
     <r>
@@ -891,19 +1122,34 @@
 1918 Part IV orchestration: 3 Flutes, 3 Oboes, 2 Clarinets, 3 Bassoons, 4 Horns, 2 Trumpets, 3 Trombones, Tuba, Xylophone, 3 Timpani, Percussion, crotales, Castanets, 2 Harps, 2 Violins, Viola, Cello, Double Bass</t>
   </si>
   <si>
+    <t>M. 44</t>
+  </si>
+  <si>
     <t>C major</t>
   </si>
   <si>
+    <t>M. 45</t>
+  </si>
+  <si>
     <t>L'aurore</t>
   </si>
   <si>
     <t>T, Mixed Choir, Orchestra</t>
   </si>
   <si>
+    <t>M. 46</t>
+  </si>
+  <si>
     <t>Introduction et allegro</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t>1. Introduction. Très lent (G</t>
     </r>
     <r>
@@ -948,6 +1194,9 @@
     <t>Harp, Flute, Clarinet, 2 Violins, Viola et Cello</t>
   </si>
   <si>
+    <t>M. 47</t>
+  </si>
+  <si>
     <t>Noël des jouets: Le troupeau verni des moutons</t>
   </si>
   <si>
@@ -955,10 +1204,19 @@
 transcription pour voix et orchestre, Ravel, 1906 révisé en 1913</t>
   </si>
   <si>
+    <t>M. 48</t>
+  </si>
+  <si>
     <t>Les grands vents d'outre-mer: Les grands vents venus d'outre-mer</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t>Modéré, très agité (E</t>
     </r>
     <r>
@@ -982,6 +1240,9 @@
   </si>
   <si>
     <t>Texte: Henri de Régnier</t>
+  </si>
+  <si>
+    <t>M. 49</t>
   </si>
   <si>
     <t>1906-1912</t>
@@ -997,10 +1258,19 @@
 [travail détruit par l'auteur]</t>
   </si>
   <si>
+    <t>M. 50</t>
+  </si>
+  <si>
     <t>Histoires naturelles</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t>1. Le paon: Il va surement se marier aujourd'hui Sans hâte et noblement (F)
 2. Le grillon: C'est l'heure où, las d'errer Placide (a)
 3. Le cygne: Il glisse sur le bassin Lent (B)
@@ -1033,16 +1303,28 @@
     <t>Texte: Jules Renard</t>
   </si>
   <si>
+    <t>M. 51</t>
+  </si>
+  <si>
     <t>Vocalise-étude en forme de habanera</t>
   </si>
   <si>
     <t>Presque lent et avec indolence (g)</t>
   </si>
   <si>
+    <t>M. 52</t>
+  </si>
+  <si>
     <t>L'heure espagnole</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t>V1, V2, V3, V4, V5, 3 Flutes, 3 Oboes, 2 Clarinets in A, Clarinet in B</t>
     </r>
     <r>
@@ -1069,10 +1351,19 @@
     <t>Livret: Franc-Nohain</t>
   </si>
   <si>
+    <t>M. 53</t>
+  </si>
+  <si>
     <t>Sur l'herbe: L'abbé divague. Et toi, marquis</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t>Modéré (c</t>
     </r>
     <r>
@@ -1095,10 +1386,19 @@
     </r>
   </si>
   <si>
+    <t>M. 54</t>
+  </si>
+  <si>
     <t>Rhapsodie espagnole, pour orchestre</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t>1. Prélude à la nuit. Très modéré (a)
 2. Malaguena. Assez vif (a)
 3. Habanera. Assez lent et d'un rythme las (f</t>
@@ -1146,10 +1446,19 @@
 1st version, 1907: 2 Pianos</t>
   </si>
   <si>
+    <t>M. 55</t>
+  </si>
+  <si>
     <t>Gaspard de la nuit</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t>1. Ondine Lent (C</t>
     </r>
     <r>
@@ -1195,6 +1504,9 @@
     <t>after Aloysius Bertrand</t>
   </si>
   <si>
+    <t>M. 56</t>
+  </si>
+  <si>
     <t>Pavane de la Belle au bois dormant</t>
   </si>
   <si>
@@ -1208,6 +1520,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Inspiré par Charles Perrault
 [Inclus comme </t>
     </r>
@@ -1249,6 +1567,9 @@
     </r>
   </si>
   <si>
+    <t>M. 57</t>
+  </si>
+  <si>
     <t>1909-1912</t>
   </si>
   <si>
@@ -1261,7 +1582,7 @@
     <t>Livret: Michel Fokine et Maurice Ravel d'après Longus</t>
   </si>
   <si>
-    <t>57a</t>
+    <t>M. 57a</t>
   </si>
   <si>
     <t>1. Nocturne, with choir a cappella or orchestration solo
@@ -1270,6 +1591,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF330000"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">suite d'orchestre </t>
     </r>
     <r>
@@ -1292,7 +1619,7 @@
     </r>
   </si>
   <si>
-    <t>57b</t>
+    <t>M. 57b</t>
   </si>
   <si>
     <t>1. Lever du jour
@@ -1303,7 +1630,7 @@
     <t>suite d'orchestre #2</t>
   </si>
   <si>
-    <t>57c</t>
+    <t>M. 57c</t>
   </si>
   <si>
     <t>Danse gracieuse de Daphnis</t>
@@ -1314,10 +1641,16 @@
 3. Scène de Daphnis et Chloé</t>
   </si>
   <si>
+    <t>M. 58</t>
+  </si>
+  <si>
     <t>Menuet sur le nom de Haydn</t>
   </si>
   <si>
     <t>pour un numéro consacré à Haydn par la Revue Musicale</t>
+  </si>
+  <si>
+    <t>M. 59</t>
   </si>
   <si>
     <t>1909-1910</t>
@@ -1333,6 +1666,9 @@
 [lost]</t>
   </si>
   <si>
+    <t>M. 60</t>
+  </si>
+  <si>
     <t>1908-1910</t>
   </si>
   <si>
@@ -1340,6 +1676,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">1. Pavane de la belle au bois dormant [de </t>
     </r>
     <r>
@@ -1388,10 +1730,19 @@
 orchestration, Ravel, 1911, O 62 ci-dessous</t>
   </si>
   <si>
+    <t>M. 61</t>
+  </si>
+  <si>
     <t>Valses nobles et sentimentales</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t>1. Modéré - très franc (G)
 2. Assez lent - avec une expression intense (g)
 3. Modéré (e)
@@ -1428,6 +1779,9 @@
     <t>transcription pour orchestre, Ravel, 1912 utilisée comme musique de ballet: Adélaïde ou le langage des fleurs</t>
   </si>
   <si>
+    <t>M. 62</t>
+  </si>
+  <si>
     <t>1911-1912</t>
   </si>
   <si>
@@ -1435,6 +1789,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t>1. Prélude
 2. Danse du rouet et scène
 3. Pavane de la belle au bois dormant(2 Flutes, Oboes, English Horn, 2 Clarinets, Bassoon, Horn, Harp, cordes) Lent (a)
@@ -1503,6 +1863,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">[Ajouts et orchestration de la suite </t>
     </r>
     <r>
@@ -1525,6 +1891,9 @@
     </r>
   </si>
   <si>
+    <t>M. 63</t>
+  </si>
+  <si>
     <t>1912-1913</t>
   </si>
   <si>
@@ -1532,6 +1901,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t>1. Borodine Valse (D</t>
     </r>
     <r>
@@ -1556,6 +1931,9 @@
   </si>
   <si>
     <t>[Pastiches suggérés par Alfredo Casella]</t>
+  </si>
+  <si>
+    <t>M. 64</t>
   </si>
   <si>
     <t>Trois poèmes de Stéphane Mallarmé</t>
@@ -1570,9 +1948,15 @@
 1913 transcription: Voice, Piano</t>
   </si>
   <si>
+    <t>M. 65</t>
+  </si>
+  <si>
     <t>Prélude</t>
   </si>
   <si>
+    <t>M. 66</t>
+  </si>
+  <si>
     <t>1913-1914</t>
   </si>
   <si>
@@ -1585,10 +1969,19 @@
     <t>[Esquisses sur des thèmes basques]</t>
   </si>
   <si>
+    <t>M. 67</t>
+  </si>
+  <si>
     <t>Trio</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t>1. Modéré (a)
 2. Pantoum. Assez vite (a)
 3. Passacaille. Très large (f</t>
@@ -1615,6 +2008,9 @@
   </si>
   <si>
     <t>Piano, Violin, Cello</t>
+  </si>
+  <si>
+    <t>M. 68</t>
   </si>
   <si>
     <t>1914-1917</t>
@@ -1631,7 +2027,7 @@
 6. Toccata Vif (e)</t>
   </si>
   <si>
-    <t>68a</t>
+    <t>M. 68.1</t>
   </si>
   <si>
     <t>1. Prélude Vif (e)
@@ -1643,6 +2039,9 @@
     <t>2 Flutes, Oboes, English Horn, 2 Clarinets, 2 Bassoons, Trumpet, Harp, 2 Violins, Viola, Cello, Double Bass</t>
   </si>
   <si>
+    <t>M. 69</t>
+  </si>
+  <si>
     <t>1914-1915</t>
   </si>
   <si>
@@ -1661,6 +2060,9 @@
     <t>Texte: Maurice Ravel</t>
   </si>
   <si>
+    <t>M. 70</t>
+  </si>
+  <si>
     <t>Frontispice</t>
   </si>
   <si>
@@ -1671,6 +2073,9 @@
   </si>
   <si>
     <t>Indicatif musical pour "S.P. 503 Le poème de Vardar" de Ricciotto Canudo</t>
+  </si>
+  <si>
+    <t>M. 71</t>
   </si>
   <si>
     <t>1919-1925</t>
@@ -1694,6 +2099,9 @@
     <t>Texte: Colette</t>
   </si>
   <si>
+    <t>M. 72</t>
+  </si>
+  <si>
     <t>1919-1920</t>
   </si>
   <si>
@@ -1709,6 +2117,9 @@
 [????] transcription: Piano Four Hands</t>
   </si>
   <si>
+    <t>M. 73</t>
+  </si>
+  <si>
     <t>1920-1922</t>
   </si>
   <si>
@@ -1724,10 +2135,16 @@
     <t>premier mouvement paru sous le titre Duo dans Le Tombeau de Claude Debussy, 1920</t>
   </si>
   <si>
+    <t>M. 74</t>
+  </si>
+  <si>
     <t>Berceuse sur le nom de Gabriel Fauré</t>
   </si>
   <si>
     <t>Simplice (G)</t>
+  </si>
+  <si>
+    <t>M. 75</t>
   </si>
   <si>
     <t>1923-1924</t>
@@ -1743,6 +2160,9 @@
     <t>Texte: Douzain de Ronsard</t>
   </si>
   <si>
+    <t>M. 76</t>
+  </si>
+  <si>
     <t>1922-1924</t>
   </si>
   <si>
@@ -1756,10 +2176,19 @@
 2. Solo Violin, 2 Flutes, 2 Oboes, 2 Clarinets, 2 Bassoons, 2 Horns, Trumpet, Triangle, Timbres, Cymbal, Celesta, Harp, 2 Violins, Viola, Cello, Double Bass</t>
   </si>
   <si>
+    <t>M. 77</t>
+  </si>
+  <si>
     <t>1923-1927</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t>1. Allegretto (G)
 2. Blues. Moderato (A</t>
     </r>
@@ -1785,6 +2214,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Sonate </t>
     </r>
     <r>
@@ -1805,6 +2240,9 @@
       </rPr>
       <t>2</t>
     </r>
+  </si>
+  <si>
+    <t>M. 78</t>
   </si>
   <si>
     <t>1925-1926</t>
@@ -1824,10 +2262,16 @@
     <t>Texte: Evariste-Désiré Parny de Forges</t>
   </si>
   <si>
+    <t>M. 79</t>
+  </si>
+  <si>
     <t>Rêves: Un enfant court</t>
   </si>
   <si>
     <t>Texte: Léon-Paul Fargue</t>
+  </si>
+  <si>
+    <t>M. 80</t>
   </si>
   <si>
     <t>Fanfare, prélude à "L'évantail de Jeanne", ballet collectif en un acte</t>
@@ -1837,6 +2281,9 @@
 1927 transcription: Piano Four Hands</t>
   </si>
   <si>
+    <t>M. 81</t>
+  </si>
+  <si>
     <t>Boléro</t>
   </si>
   <si>
@@ -1847,6 +2294,9 @@
   </si>
   <si>
     <t>transcription pour piano deux mains et quatre mains, Ravel, 1929</t>
+  </si>
+  <si>
+    <t>M. 82</t>
   </si>
   <si>
     <t>1929-1930</t>
@@ -1864,6 +2314,9 @@
   <si>
     <t>[Commande du pianiste Paul Wittgenstein]
 réduction pour piano de la partie orchestre, Ravel, 1930</t>
+  </si>
+  <si>
+    <t>M. 83</t>
   </si>
   <si>
     <t>1929-1931</t>
@@ -1880,6 +2333,9 @@
     <t>transcription pour deux pianos (réduction de l'orchestre au 2è piano), Ravel, 1932</t>
   </si>
   <si>
+    <t>M. 84</t>
+  </si>
+  <si>
     <t>1932-1933</t>
   </si>
   <si>
@@ -1887,6 +2343,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="OPPO Sans 4.0"/>
+        <charset val="134"/>
+      </rPr>
       <t>1. Chanson romanesque: Si vous me disiez que la terre Moderato (b</t>
     </r>
     <r>
@@ -1934,6 +2396,9 @@
   <si>
     <t>Texte: Paul Morand
 transcription pour baryton et piano, Ravel, 1933</t>
+  </si>
+  <si>
+    <t>M. 85</t>
   </si>
   <si>
     <t>Morgiane</t>
@@ -3158,17 +3623,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G92"/>
-  <sheetFormatPr defaultColWidth="8.61261261261261" defaultRowHeight="30" customHeight="1" outlineLevelCol="6"/>
+  <dimension ref="A1:I92"/>
+  <sheetFormatPr defaultColWidth="8.61261261261261" defaultRowHeight="30" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="14.4414414414414" style="3" customWidth="1"/>
-    <col min="3" max="3" width="23.7027027027027" style="4" customWidth="1"/>
-    <col min="4" max="4" width="14.5855855855856" style="3" customWidth="1"/>
-    <col min="5" max="7" width="23.7027027027027" style="5" customWidth="1"/>
-    <col min="8" max="16384" width="8.61261261261261" style="2"/>
+    <col min="1" max="3" width="14.4414414414414" style="3" customWidth="1"/>
+    <col min="4" max="4" width="23.7027027027027" style="4" customWidth="1"/>
+    <col min="5" max="5" width="14.5855855855856" style="3" customWidth="1"/>
+    <col min="6" max="8" width="23.7027027027027" style="5" customWidth="1"/>
+    <col min="9" max="16384" width="8.61261261261261" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" customHeight="1" spans="1:7">
+    <row r="1" s="1" customFormat="1" customHeight="1" spans="1:9">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -3184,1845 +3649,2117 @@
       <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="H1" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" s="2" customFormat="1" customHeight="1" spans="1:9">
       <c r="A2" s="8">
         <v>1</v>
       </c>
-      <c r="B2" s="8">
+      <c r="B2" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="8">
         <v>1888</v>
       </c>
-      <c r="C2" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="8"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="10" t="s">
-        <v>8</v>
-      </c>
+      <c r="D2" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="8"/>
+      <c r="F2" s="9"/>
       <c r="G2" s="10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>10</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" s="2" customFormat="1" customHeight="1" spans="1:9">
       <c r="A3" s="8">
         <v>2</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="8">
         <v>1888</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="D3" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="8"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="8"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="H3" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" s="2" customFormat="1" customHeight="1" spans="1:9">
       <c r="A4" s="8">
         <v>3</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="8">
         <v>1888</v>
       </c>
-      <c r="C4" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="8"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="10" t="s">
-        <v>8</v>
-      </c>
+      <c r="D4" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="8"/>
+      <c r="F4" s="9"/>
       <c r="G4" s="10" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>10</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" s="2" customFormat="1" customHeight="1" spans="1:9">
       <c r="A5" s="8">
         <v>4</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="8">
         <v>1893</v>
       </c>
-      <c r="C5" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="F5" s="10" t="s">
-        <v>17</v>
+      <c r="D5" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>23</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" s="2" customFormat="1" customHeight="1" spans="1:9">
       <c r="A6" s="8">
         <v>5</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" s="8"/>
-      <c r="E6" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="F6" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="G6" s="10"/>
-    </row>
-    <row r="7" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>25</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="8"/>
+      <c r="F6" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="H6" s="10"/>
+    </row>
+    <row r="7" s="2" customFormat="1" customHeight="1" spans="1:9">
       <c r="A7" s="8">
         <v>6</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="8">
         <v>1895</v>
       </c>
-      <c r="C7" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D7" s="8"/>
-      <c r="E7" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>25</v>
+      <c r="D7" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="8"/>
+      <c r="F7" s="9" t="s">
+        <v>32</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="8" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>33</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" s="2" customFormat="1" customHeight="1" spans="1:9">
       <c r="A8" s="8">
         <v>7</v>
       </c>
-      <c r="B8" s="8">
+      <c r="B8" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="8">
         <v>1895</v>
       </c>
-      <c r="C8" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E8" s="9" t="s">
+      <c r="D8" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="G8" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="F8" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="H8" s="10" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" s="2" customFormat="1" customHeight="1" spans="1:9">
       <c r="A9" s="8">
         <v>8</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="8">
         <v>1895</v>
       </c>
-      <c r="C9" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="D9" s="8"/>
-      <c r="E9" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="F9" s="10" t="s">
-        <v>33</v>
+      <c r="D9" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E9" s="8"/>
+      <c r="F9" s="9" t="s">
+        <v>42</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="10" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>43</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" s="2" customFormat="1" customHeight="1" spans="1:9">
       <c r="A10" s="8">
         <v>9</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="8">
         <v>1896</v>
       </c>
-      <c r="C10" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>38</v>
+      <c r="D10" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>48</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="11" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>49</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" s="2" customFormat="1" customHeight="1" spans="1:9">
       <c r="A11" s="8">
         <v>10</v>
       </c>
-      <c r="B11" s="8">
+      <c r="B11" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="8">
         <v>1896</v>
       </c>
-      <c r="C11" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F11" s="10" t="s">
-        <v>43</v>
+      <c r="D11" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>54</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="12" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>55</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" s="2" customFormat="1" customHeight="1" spans="1:9">
       <c r="A12" s="8">
         <v>11</v>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C12" s="8">
         <v>1896</v>
       </c>
-      <c r="C12" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="D12" s="8"/>
-      <c r="E12" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="F12" s="10" t="s">
-        <v>8</v>
+      <c r="D12" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="E12" s="8"/>
+      <c r="F12" s="9" t="s">
+        <v>59</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="13" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>10</v>
+      </c>
+      <c r="H12" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" s="2" customFormat="1" customHeight="1" spans="1:9">
       <c r="A13" s="8">
         <v>12</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" s="8">
         <v>1897</v>
       </c>
-      <c r="C13" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="D13" s="8"/>
-      <c r="E13" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="F13" s="10" t="s">
-        <v>50</v>
+      <c r="D13" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="E13" s="8"/>
+      <c r="F13" s="9" t="s">
+        <v>63</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="14" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>64</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="14" s="2" customFormat="1" customHeight="1" spans="1:9">
       <c r="A14" s="8">
         <v>13</v>
       </c>
-      <c r="B14" s="8">
+      <c r="B14" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="8">
         <v>1897</v>
       </c>
-      <c r="C14" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="F14" s="10" t="s">
-        <v>33</v>
+      <c r="D14" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>69</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="15" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>43</v>
+      </c>
+      <c r="H14" s="10" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="15" s="2" customFormat="1" customHeight="1" spans="1:9">
       <c r="A15" s="8">
         <v>14</v>
       </c>
-      <c r="B15" s="8">
+      <c r="B15" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C15" s="8">
         <v>1898</v>
       </c>
-      <c r="C15" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="F15" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="G15" s="10"/>
-    </row>
-    <row r="16" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="D15" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H15" s="10"/>
+    </row>
+    <row r="16" s="2" customFormat="1" customHeight="1" spans="1:9">
       <c r="A16" s="8">
         <v>15</v>
       </c>
-      <c r="B16" s="8">
+      <c r="B16" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C16" s="8">
         <v>1898</v>
       </c>
-      <c r="C16" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="D16" s="8"/>
-      <c r="E16" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="F16" s="10" t="s">
-        <v>17</v>
+      <c r="D16" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="E16" s="8"/>
+      <c r="F16" s="9" t="s">
+        <v>77</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="17" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>23</v>
+      </c>
+      <c r="H16" s="10" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="17" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A17" s="8">
         <v>16</v>
       </c>
-      <c r="B17" s="8">
+      <c r="B17" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C17" s="8">
         <v>1898</v>
       </c>
-      <c r="C17" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="D17" s="8"/>
-      <c r="E17" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="F17" s="10" t="s">
-        <v>17</v>
+      <c r="D17" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="E17" s="8"/>
+      <c r="F17" s="9" t="s">
+        <v>77</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="18" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>23</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="18" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A18" s="8">
         <v>17</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B18" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="C18" s="8">
         <v>1898</v>
       </c>
-      <c r="C18" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="D18" s="8"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="10" t="s">
-        <v>65</v>
-      </c>
+      <c r="D18" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="E18" s="8"/>
+      <c r="F18" s="9"/>
       <c r="G18" s="10" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="19" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>84</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="19" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A19" s="8">
         <v>18</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="D19" s="8"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="10" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="20" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>86</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="E19" s="8"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="20" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A20" s="8">
         <v>19</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B20" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="C20" s="8">
         <v>1899</v>
       </c>
-      <c r="C20" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="E20" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="F20" s="10" t="s">
-        <v>8</v>
+      <c r="D20" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>93</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="21" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>10</v>
+      </c>
+      <c r="H20" s="10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="21" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A21" s="8">
         <v>20</v>
       </c>
-      <c r="B21" s="8">
+      <c r="B21" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="C21" s="8">
         <v>1899</v>
       </c>
-      <c r="C21" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="D21" s="8"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="22" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="D21" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="E21" s="8"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="10" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="22" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A22" s="8">
         <v>21</v>
       </c>
-      <c r="B22" s="8">
+      <c r="B22" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C22" s="8">
         <v>1899</v>
       </c>
-      <c r="C22" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="D22" s="8"/>
-      <c r="E22" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="F22" s="10" t="s">
-        <v>17</v>
+      <c r="D22" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="E22" s="8"/>
+      <c r="F22" s="9" t="s">
+        <v>100</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="23" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>23</v>
+      </c>
+      <c r="H22" s="10" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="23" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A23" s="8">
         <v>22</v>
       </c>
-      <c r="B23" s="8">
+      <c r="B23" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="C23" s="8">
         <v>1900</v>
       </c>
-      <c r="C23" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="D23" s="8"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="10"/>
-      <c r="G23" s="10" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="24" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="D23" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="E23" s="8"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="24" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A24" s="8">
         <v>23</v>
       </c>
-      <c r="B24" s="8">
+      <c r="B24" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="C24" s="8">
         <v>1900</v>
       </c>
-      <c r="C24" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="D24" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="E24" s="9"/>
-      <c r="F24" s="10" t="s">
-        <v>8</v>
-      </c>
+      <c r="D24" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="F24" s="9"/>
       <c r="G24" s="10" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="25" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>10</v>
+      </c>
+      <c r="H24" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="25" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A25" s="8">
         <v>24</v>
       </c>
-      <c r="B25" s="8">
+      <c r="B25" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="C25" s="8">
         <v>1900</v>
       </c>
-      <c r="C25" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="D25" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="E25" s="9"/>
-      <c r="F25" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="G25" s="10"/>
-    </row>
-    <row r="26" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="D25" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="F25" s="9"/>
+      <c r="G25" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H25" s="10"/>
+    </row>
+    <row r="26" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A26" s="8">
         <v>25</v>
       </c>
-      <c r="B26" s="8">
+      <c r="B26" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C26" s="8">
         <v>1900</v>
       </c>
-      <c r="C26" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="D26" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="E26" s="9"/>
-      <c r="F26" s="10" t="s">
-        <v>85</v>
-      </c>
+      <c r="D26" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="F26" s="9"/>
       <c r="G26" s="10" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="27" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>112</v>
+      </c>
+      <c r="H26" s="10" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="27" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A27" s="8">
         <v>26</v>
       </c>
-      <c r="B27" s="8">
+      <c r="B27" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C27" s="8">
         <v>1900</v>
       </c>
-      <c r="C27" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="D27" s="8"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="10" t="s">
-        <v>8</v>
-      </c>
+      <c r="D27" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="E27" s="8"/>
+      <c r="F27" s="9"/>
       <c r="G27" s="10" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="28" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>10</v>
+      </c>
+      <c r="H27" s="10" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="28" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A28" s="8">
         <v>27</v>
       </c>
-      <c r="B28" s="8">
+      <c r="B28" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="C28" s="8">
         <v>1900</v>
       </c>
-      <c r="C28" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="D28" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="E28" s="9"/>
-      <c r="F28" s="10" t="s">
-        <v>8</v>
-      </c>
+      <c r="D28" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="F28" s="9"/>
       <c r="G28" s="10" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="29" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>10</v>
+      </c>
+      <c r="H28" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="29" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A29" s="8">
         <v>28</v>
       </c>
-      <c r="B29" s="8">
+      <c r="B29" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="C29" s="8">
         <v>1901</v>
       </c>
-      <c r="C29" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="D29" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="E29" s="9"/>
-      <c r="F29" s="10" t="s">
-        <v>85</v>
-      </c>
+      <c r="D29" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="F29" s="9"/>
       <c r="G29" s="10" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="30" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>112</v>
+      </c>
+      <c r="H29" s="10" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="30" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A30" s="8">
         <v>29</v>
       </c>
-      <c r="B30" s="8">
+      <c r="B30" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="C30" s="8">
         <v>1901</v>
       </c>
-      <c r="C30" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="D30" s="8"/>
-      <c r="E30" s="9"/>
-      <c r="F30" s="10" t="s">
-        <v>93</v>
-      </c>
+      <c r="D30" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="E30" s="8"/>
+      <c r="F30" s="9"/>
       <c r="G30" s="10" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="31" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>124</v>
+      </c>
+      <c r="H30" s="10" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="31" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A31" s="8">
         <v>30</v>
       </c>
-      <c r="B31" s="8">
+      <c r="B31" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="C31" s="8">
         <v>1901</v>
       </c>
-      <c r="C31" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="D31" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="E31" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="F31" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="G31" s="10"/>
-    </row>
-    <row r="32" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="D31" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="G31" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H31" s="10"/>
+    </row>
+    <row r="32" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A32" s="8">
         <v>31</v>
       </c>
-      <c r="B32" s="8">
+      <c r="B32" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="C32" s="8">
         <v>1902</v>
       </c>
-      <c r="C32" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="D32" s="8"/>
-      <c r="E32" s="9"/>
-      <c r="F32" s="10"/>
-      <c r="G32" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="33" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="D32" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="E32" s="8"/>
+      <c r="F32" s="9"/>
+      <c r="G32" s="10"/>
+      <c r="H32" s="10" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="33" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A33" s="8">
         <v>32</v>
       </c>
-      <c r="B33" s="8">
+      <c r="B33" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="C33" s="8">
         <v>1902</v>
       </c>
-      <c r="C33" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="D33" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="E33" s="9"/>
-      <c r="F33" s="10" t="s">
-        <v>8</v>
-      </c>
+      <c r="D33" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="F33" s="9"/>
       <c r="G33" s="10" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="34" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>10</v>
+      </c>
+      <c r="H33" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="34" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A34" s="8">
         <v>33</v>
       </c>
-      <c r="B34" s="8">
+      <c r="B34" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="C34" s="8">
         <v>1902</v>
       </c>
-      <c r="C34" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="D34" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="E34" s="9"/>
-      <c r="F34" s="10" t="s">
-        <v>85</v>
-      </c>
+      <c r="D34" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="F34" s="9"/>
       <c r="G34" s="10" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="35" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>112</v>
+      </c>
+      <c r="H34" s="10" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="35" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A35" s="8">
         <v>34</v>
       </c>
-      <c r="B35" s="8">
+      <c r="B35" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="C35" s="8">
         <v>1902</v>
       </c>
-      <c r="C35" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="D35" s="8"/>
-      <c r="E35" s="9"/>
-      <c r="F35" s="10"/>
-      <c r="G35" s="10" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="36" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="D35" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="E35" s="8"/>
+      <c r="F35" s="9"/>
+      <c r="G35" s="10"/>
+      <c r="H35" s="10" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="36" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A36" s="8">
         <v>35</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="C36" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="D36" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="E36" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="F36" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="G36" s="10"/>
-    </row>
-    <row r="37" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>140</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="E36" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="F36" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="G36" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="H36" s="10"/>
+    </row>
+    <row r="37" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A37" s="8">
         <v>36</v>
       </c>
-      <c r="B37" s="8">
+      <c r="B37" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="C37" s="8">
         <v>1903</v>
       </c>
-      <c r="C37" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="D37" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E37" s="9"/>
-      <c r="F37" s="10" t="s">
-        <v>8</v>
-      </c>
+      <c r="D37" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="E37" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="F37" s="9"/>
       <c r="G37" s="10" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="38" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>10</v>
+      </c>
+      <c r="H37" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="38" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A38" s="8">
         <v>37</v>
       </c>
-      <c r="B38" s="8">
+      <c r="B38" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="C38" s="8">
         <v>1903</v>
       </c>
-      <c r="C38" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="D38" s="8"/>
-      <c r="E38" s="9"/>
-      <c r="F38" s="10" t="s">
-        <v>110</v>
-      </c>
+      <c r="D38" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="E38" s="8"/>
+      <c r="F38" s="9"/>
       <c r="G38" s="10" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="39" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>149</v>
+      </c>
+      <c r="H38" s="10" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="39" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A39" s="8">
         <v>38</v>
       </c>
-      <c r="B39" s="8">
+      <c r="B39" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="C39" s="8">
         <v>1903</v>
       </c>
-      <c r="C39" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="D39" s="8"/>
-      <c r="E39" s="9"/>
-      <c r="F39" s="10" t="s">
-        <v>93</v>
-      </c>
+      <c r="D39" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="E39" s="8"/>
+      <c r="F39" s="9"/>
       <c r="G39" s="10" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="40" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>124</v>
+      </c>
+      <c r="H39" s="10" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="40" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A40" s="8">
         <v>39</v>
       </c>
-      <c r="B40" s="8">
+      <c r="B40" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="C40" s="8">
         <v>1903</v>
       </c>
-      <c r="C40" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="D40" s="8"/>
-      <c r="E40" s="9"/>
-      <c r="F40" s="10" t="s">
-        <v>17</v>
-      </c>
+      <c r="D40" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="E40" s="8"/>
+      <c r="F40" s="9"/>
       <c r="G40" s="10" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="41" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>23</v>
+      </c>
+      <c r="H40" s="10" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="41" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A41" s="8">
         <v>40</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="C41" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="D41" s="8"/>
-      <c r="E41" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="F41" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="G41" s="10"/>
-    </row>
-    <row r="42" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>156</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="D41" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="E41" s="8"/>
+      <c r="F41" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="G41" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H41" s="10"/>
+    </row>
+    <row r="42" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A42" s="8">
         <v>41</v>
       </c>
-      <c r="B42" s="8">
+      <c r="B42" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="C42" s="8">
         <v>1903</v>
       </c>
-      <c r="C42" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="D42" s="8"/>
-      <c r="E42" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="F42" s="10" t="s">
-        <v>119</v>
+      <c r="D42" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="E42" s="8"/>
+      <c r="F42" s="9" t="s">
+        <v>161</v>
       </c>
       <c r="G42" s="10" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="43" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>162</v>
+      </c>
+      <c r="H42" s="10" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="43" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A43" s="8">
         <v>42</v>
       </c>
-      <c r="B43" s="8">
+      <c r="B43" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="C43" s="8">
         <v>1904</v>
       </c>
-      <c r="C43" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="D43" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="E43" s="9"/>
-      <c r="F43" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="G43" s="10"/>
-    </row>
-    <row r="44" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="D43" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="E43" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="F43" s="9"/>
+      <c r="G43" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H43" s="10"/>
+    </row>
+    <row r="44" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A44" s="8">
         <v>43</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="C44" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="D44" s="8"/>
-      <c r="E44" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="F44" s="10" t="s">
-        <v>125</v>
-      </c>
-      <c r="G44" s="10"/>
-    </row>
-    <row r="45" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>166</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="D44" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="E44" s="8"/>
+      <c r="F44" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="G44" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="H44" s="10"/>
+    </row>
+    <row r="45" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A45" s="8">
         <v>44</v>
       </c>
-      <c r="B45" s="8">
+      <c r="B45" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="C45" s="8">
         <v>1905</v>
       </c>
-      <c r="C45" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="D45" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="E45" s="9"/>
-      <c r="F45" s="10" t="s">
-        <v>8</v>
-      </c>
+      <c r="D45" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="E45" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="F45" s="9"/>
       <c r="G45" s="10" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="46" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>10</v>
+      </c>
+      <c r="H45" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="46" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A46" s="8">
         <v>45</v>
       </c>
-      <c r="B46" s="8">
+      <c r="B46" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="C46" s="8">
         <v>1905</v>
       </c>
-      <c r="C46" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="D46" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="E46" s="9"/>
-      <c r="F46" s="10" t="s">
-        <v>128</v>
-      </c>
+      <c r="D46" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="E46" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="F46" s="9"/>
       <c r="G46" s="10" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="47" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>175</v>
+      </c>
+      <c r="H46" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="47" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A47" s="8">
         <v>46</v>
       </c>
-      <c r="B47" s="8">
+      <c r="B47" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="C47" s="8">
         <v>1905</v>
       </c>
-      <c r="C47" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="D47" s="8"/>
-      <c r="E47" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="F47" s="10" t="s">
-        <v>131</v>
-      </c>
-      <c r="G47" s="10"/>
-    </row>
-    <row r="48" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="D47" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="E47" s="8"/>
+      <c r="F47" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="G47" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="H47" s="10"/>
+    </row>
+    <row r="48" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A48" s="8">
         <v>47</v>
       </c>
-      <c r="B48" s="8">
+      <c r="B48" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="C48" s="8">
         <v>1905</v>
       </c>
-      <c r="C48" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="D48" s="8"/>
-      <c r="E48" s="9"/>
-      <c r="F48" s="10" t="s">
-        <v>17</v>
-      </c>
+      <c r="D48" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="E48" s="8"/>
+      <c r="F48" s="9"/>
       <c r="G48" s="10" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="49" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>23</v>
+      </c>
+      <c r="H48" s="10" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="49" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A49" s="8">
         <v>48</v>
       </c>
-      <c r="B49" s="8">
+      <c r="B49" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="C49" s="8">
         <v>1906</v>
       </c>
-      <c r="C49" s="9" t="s">
+      <c r="D49" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="E49" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="D49" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="E49" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="F49" s="10" t="s">
-        <v>17</v>
+      <c r="F49" s="9" t="s">
+        <v>185</v>
       </c>
       <c r="G49" s="10" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="50" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>23</v>
+      </c>
+      <c r="H49" s="10" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="50" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A50" s="8">
         <v>49</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="C50" s="9" t="s">
-        <v>138</v>
-      </c>
-      <c r="D50" s="8"/>
-      <c r="E50" s="9"/>
-      <c r="F50" s="10" t="s">
-        <v>139</v>
-      </c>
+        <v>187</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>188</v>
+      </c>
+      <c r="D50" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="E50" s="8"/>
+      <c r="F50" s="9"/>
       <c r="G50" s="10" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="51" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>190</v>
+      </c>
+      <c r="H50" s="10" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="51" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A51" s="8">
         <v>50</v>
       </c>
-      <c r="B51" s="8">
+      <c r="B51" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="C51" s="8">
         <v>1906</v>
       </c>
-      <c r="C51" s="9" t="s">
-        <v>141</v>
-      </c>
-      <c r="D51" s="8"/>
-      <c r="E51" s="9" t="s">
-        <v>142</v>
-      </c>
-      <c r="F51" s="10" t="s">
-        <v>143</v>
+      <c r="D51" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="E51" s="8"/>
+      <c r="F51" s="9" t="s">
+        <v>194</v>
       </c>
       <c r="G51" s="10" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="52" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>195</v>
+      </c>
+      <c r="H51" s="10" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="52" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A52" s="8">
         <v>51</v>
       </c>
-      <c r="B52" s="8">
+      <c r="B52" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="C52" s="8">
         <v>1907</v>
       </c>
-      <c r="C52" s="9" t="s">
-        <v>145</v>
-      </c>
-      <c r="D52" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="E52" s="9" t="s">
-        <v>146</v>
-      </c>
-      <c r="F52" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="G52" s="10"/>
-    </row>
-    <row r="53" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="D52" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="E52" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="F52" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="G52" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="H52" s="10"/>
+    </row>
+    <row r="53" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A53" s="8">
         <v>52</v>
       </c>
-      <c r="B53" s="8">
+      <c r="B53" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="C53" s="8">
         <v>1907</v>
       </c>
-      <c r="C53" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="D53" s="8"/>
-      <c r="E53" s="9"/>
-      <c r="F53" s="10" t="s">
-        <v>148</v>
-      </c>
+      <c r="D53" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="E53" s="8"/>
+      <c r="F53" s="9"/>
       <c r="G53" s="10" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="54" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>202</v>
+      </c>
+      <c r="H53" s="10" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="54" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A54" s="8">
         <v>53</v>
       </c>
-      <c r="B54" s="8">
+      <c r="B54" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="C54" s="8">
         <v>1907</v>
       </c>
-      <c r="C54" s="9" t="s">
-        <v>150</v>
-      </c>
-      <c r="D54" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="E54" s="9" t="s">
-        <v>151</v>
-      </c>
-      <c r="F54" s="10" t="s">
-        <v>17</v>
+      <c r="D54" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="E54" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="F54" s="9" t="s">
+        <v>206</v>
       </c>
       <c r="G54" s="10" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="55" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>23</v>
+      </c>
+      <c r="H54" s="10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="55" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A55" s="8">
         <v>54</v>
       </c>
-      <c r="B55" s="8">
+      <c r="B55" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="C55" s="8">
         <v>1907</v>
       </c>
-      <c r="C55" s="9" t="s">
-        <v>152</v>
-      </c>
-      <c r="D55" s="8"/>
-      <c r="E55" s="9" t="s">
-        <v>153</v>
-      </c>
-      <c r="F55" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="G55" s="10"/>
-    </row>
-    <row r="56" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="D55" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="E55" s="8"/>
+      <c r="F55" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="G55" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="H55" s="10"/>
+    </row>
+    <row r="56" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A56" s="8">
         <v>55</v>
       </c>
-      <c r="B56" s="8">
+      <c r="B56" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="C56" s="8">
         <v>1908</v>
       </c>
-      <c r="C56" s="9" t="s">
-        <v>155</v>
-      </c>
-      <c r="D56" s="8"/>
-      <c r="E56" s="9" t="s">
-        <v>156</v>
-      </c>
-      <c r="F56" s="10" t="s">
-        <v>8</v>
+      <c r="D56" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="E56" s="8"/>
+      <c r="F56" s="9" t="s">
+        <v>213</v>
       </c>
       <c r="G56" s="10" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="57" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>10</v>
+      </c>
+      <c r="H56" s="10" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="57" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A57" s="8">
         <v>56</v>
       </c>
-      <c r="B57" s="8">
+      <c r="B57" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="C57" s="8">
         <v>1908</v>
       </c>
-      <c r="C57" s="9" t="s">
-        <v>158</v>
-      </c>
-      <c r="D57" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="E57" s="9" t="s">
-        <v>160</v>
-      </c>
-      <c r="F57" s="10" t="s">
-        <v>161</v>
+      <c r="D57" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="E57" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="F57" s="9" t="s">
+        <v>218</v>
       </c>
       <c r="G57" s="10" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="58" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>219</v>
+      </c>
+      <c r="H57" s="10" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="58" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A58" s="8">
         <v>57</v>
       </c>
       <c r="B58" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="C58" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="D58" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="E58" s="9"/>
-      <c r="F58" s="10" t="s">
-        <v>165</v>
-      </c>
+        <v>221</v>
+      </c>
+      <c r="C58" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="D58" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="E58" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="F58" s="9"/>
       <c r="G58" s="10" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="59" s="2" customFormat="1" customHeight="1" spans="1:7">
-      <c r="A59" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="B59" s="8">
+        <v>224</v>
+      </c>
+      <c r="H58" s="10" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="59" s="2" customFormat="1" customHeight="1" spans="1:8">
+      <c r="A59" s="8">
+        <v>57.1</v>
+      </c>
+      <c r="B59" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="C59" s="8">
         <v>1911</v>
       </c>
-      <c r="C59" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="D59" s="8"/>
-      <c r="E59" s="9" t="s">
-        <v>168</v>
-      </c>
-      <c r="F59" s="12"/>
-      <c r="G59" s="13" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="60" s="2" customFormat="1" customHeight="1" spans="1:7">
-      <c r="A60" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="B60" s="8">
+      <c r="D59" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="E59" s="8"/>
+      <c r="F59" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="G59" s="12"/>
+      <c r="H59" s="13" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="60" s="2" customFormat="1" customHeight="1" spans="1:8">
+      <c r="A60" s="8">
+        <v>57.2</v>
+      </c>
+      <c r="B60" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="C60" s="8">
         <v>1913</v>
       </c>
-      <c r="C60" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="D60" s="8"/>
-      <c r="E60" s="9" t="s">
-        <v>171</v>
-      </c>
-      <c r="F60" s="12"/>
-      <c r="G60" s="13" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="61" s="2" customFormat="1" customHeight="1" spans="1:7">
-      <c r="A61" s="8" t="s">
-        <v>173</v>
-      </c>
-      <c r="B61" s="8">
+      <c r="D60" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="E60" s="8"/>
+      <c r="F60" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="G60" s="12"/>
+      <c r="H60" s="13" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="61" s="2" customFormat="1" customHeight="1" spans="1:8">
+      <c r="A61" s="8">
+        <v>57.3</v>
+      </c>
+      <c r="B61" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="C61" s="8">
         <v>1913</v>
       </c>
-      <c r="C61" s="9" t="s">
-        <v>174</v>
-      </c>
-      <c r="D61" s="8"/>
-      <c r="E61" s="9" t="s">
-        <v>175</v>
-      </c>
-      <c r="F61" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="G61" s="10"/>
-    </row>
-    <row r="62" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="D61" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="E61" s="8"/>
+      <c r="F61" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="G61" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H61" s="10"/>
+    </row>
+    <row r="62" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A62" s="8">
         <v>58</v>
       </c>
-      <c r="B62" s="8">
+      <c r="B62" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="C62" s="8">
         <v>1909</v>
       </c>
-      <c r="C62" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="D62" s="8"/>
-      <c r="E62" s="9"/>
-      <c r="F62" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="G62" s="13" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="63" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="D62" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="E62" s="8"/>
+      <c r="F62" s="9"/>
+      <c r="G62" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H62" s="13" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="63" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A63" s="8">
         <v>59</v>
       </c>
       <c r="B63" s="8" t="s">
-        <v>178</v>
-      </c>
-      <c r="C63" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="D63" s="8"/>
-      <c r="E63" s="9"/>
-      <c r="F63" s="10" t="s">
-        <v>180</v>
-      </c>
+        <v>238</v>
+      </c>
+      <c r="C63" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="D63" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="E63" s="8"/>
+      <c r="F63" s="9"/>
       <c r="G63" s="10" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="64" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>241</v>
+      </c>
+      <c r="H63" s="10" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="64" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A64" s="8">
         <v>60</v>
       </c>
       <c r="B64" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="C64" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="D64" s="8"/>
-      <c r="E64" s="9" t="s">
-        <v>184</v>
-      </c>
-      <c r="F64" s="10" t="s">
-        <v>161</v>
+        <v>243</v>
+      </c>
+      <c r="C64" s="8" t="s">
+        <v>244</v>
+      </c>
+      <c r="D64" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="E64" s="8"/>
+      <c r="F64" s="9" t="s">
+        <v>246</v>
       </c>
       <c r="G64" s="10" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="65" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>219</v>
+      </c>
+      <c r="H64" s="10" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="65" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A65" s="8">
         <v>61</v>
       </c>
-      <c r="B65" s="8">
+      <c r="B65" s="8" t="s">
+        <v>248</v>
+      </c>
+      <c r="C65" s="8">
         <v>1911</v>
       </c>
-      <c r="C65" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="D65" s="8"/>
-      <c r="E65" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="F65" s="10" t="s">
-        <v>188</v>
+      <c r="D65" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="E65" s="8"/>
+      <c r="F65" s="9" t="s">
+        <v>250</v>
       </c>
       <c r="G65" s="10" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="66" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>251</v>
+      </c>
+      <c r="H65" s="10" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="66" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A66" s="8">
         <v>62</v>
       </c>
       <c r="B66" s="8" t="s">
-        <v>190</v>
-      </c>
-      <c r="C66" s="9" t="s">
-        <v>191</v>
-      </c>
-      <c r="D66" s="8"/>
-      <c r="E66" s="9" t="s">
-        <v>192</v>
-      </c>
-      <c r="F66" s="10" t="s">
-        <v>193</v>
+        <v>253</v>
+      </c>
+      <c r="C66" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="D66" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="E66" s="8"/>
+      <c r="F66" s="9" t="s">
+        <v>256</v>
       </c>
       <c r="G66" s="10" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="67" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>257</v>
+      </c>
+      <c r="H66" s="10" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="67" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A67" s="8">
         <v>63</v>
       </c>
       <c r="B67" s="8" t="s">
-        <v>195</v>
-      </c>
-      <c r="C67" s="9" t="s">
-        <v>196</v>
-      </c>
-      <c r="D67" s="8"/>
-      <c r="E67" s="9" t="s">
-        <v>197</v>
-      </c>
-      <c r="F67" s="10" t="s">
-        <v>8</v>
+        <v>259</v>
+      </c>
+      <c r="C67" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="D67" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="E67" s="8"/>
+      <c r="F67" s="9" t="s">
+        <v>262</v>
       </c>
       <c r="G67" s="10" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="68" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>10</v>
+      </c>
+      <c r="H67" s="10" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="68" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A68" s="8">
         <v>64</v>
       </c>
-      <c r="B68" s="8">
+      <c r="B68" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="C68" s="8">
         <v>1913</v>
       </c>
-      <c r="C68" s="9" t="s">
-        <v>199</v>
-      </c>
-      <c r="D68" s="8"/>
-      <c r="E68" s="9" t="s">
-        <v>200</v>
-      </c>
-      <c r="F68" s="10" t="s">
-        <v>201</v>
+      <c r="D68" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="E68" s="8"/>
+      <c r="F68" s="9" t="s">
+        <v>266</v>
       </c>
       <c r="G68" s="10" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="69" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>267</v>
+      </c>
+      <c r="H68" s="10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="69" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A69" s="8">
         <v>65</v>
       </c>
-      <c r="B69" s="8">
+      <c r="B69" s="8" t="s">
+        <v>268</v>
+      </c>
+      <c r="C69" s="8">
         <v>1913</v>
       </c>
-      <c r="C69" s="9" t="s">
-        <v>202</v>
-      </c>
-      <c r="D69" s="8"/>
-      <c r="E69" s="9"/>
-      <c r="F69" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="G69" s="10"/>
-    </row>
-    <row r="70" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="D69" s="9" t="s">
+        <v>269</v>
+      </c>
+      <c r="E69" s="8"/>
+      <c r="F69" s="9"/>
+      <c r="G69" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H69" s="10"/>
+    </row>
+    <row r="70" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A70" s="8">
         <v>66</v>
       </c>
       <c r="B70" s="8" t="s">
-        <v>203</v>
-      </c>
-      <c r="C70" s="9" t="s">
-        <v>204</v>
-      </c>
-      <c r="D70" s="8"/>
-      <c r="E70" s="9"/>
-      <c r="F70" s="10" t="s">
-        <v>205</v>
-      </c>
+        <v>270</v>
+      </c>
+      <c r="C70" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="D70" s="9" t="s">
+        <v>272</v>
+      </c>
+      <c r="E70" s="8"/>
+      <c r="F70" s="9"/>
       <c r="G70" s="10" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="71" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>273</v>
+      </c>
+      <c r="H70" s="10" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="71" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A71" s="8">
         <v>67</v>
       </c>
-      <c r="B71" s="8">
+      <c r="B71" s="8" t="s">
+        <v>275</v>
+      </c>
+      <c r="C71" s="8">
         <v>1914</v>
       </c>
-      <c r="C71" s="11" t="s">
-        <v>207</v>
-      </c>
-      <c r="D71" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="E71" s="9" t="s">
-        <v>208</v>
-      </c>
-      <c r="F71" s="10" t="s">
-        <v>209</v>
-      </c>
-      <c r="G71" s="10"/>
-    </row>
-    <row r="72" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="D71" s="11" t="s">
+        <v>276</v>
+      </c>
+      <c r="E71" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="F71" s="9" t="s">
+        <v>277</v>
+      </c>
+      <c r="G71" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="H71" s="10"/>
+    </row>
+    <row r="72" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A72" s="8">
         <v>68</v>
       </c>
       <c r="B72" s="8" t="s">
-        <v>210</v>
-      </c>
-      <c r="C72" s="9" t="s">
-        <v>211</v>
-      </c>
-      <c r="D72" s="8"/>
-      <c r="E72" s="9" t="s">
-        <v>212</v>
-      </c>
-      <c r="F72" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="G72" s="10"/>
-    </row>
-    <row r="73" s="2" customFormat="1" customHeight="1" spans="1:7">
-      <c r="A73" s="8" t="s">
-        <v>213</v>
-      </c>
-      <c r="B73" s="8">
+        <v>279</v>
+      </c>
+      <c r="C72" s="8" t="s">
+        <v>280</v>
+      </c>
+      <c r="D72" s="9" t="s">
+        <v>281</v>
+      </c>
+      <c r="E72" s="8"/>
+      <c r="F72" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="G72" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H72" s="10"/>
+    </row>
+    <row r="73" s="2" customFormat="1" customHeight="1" spans="1:8">
+      <c r="A73" s="8">
+        <v>68.1</v>
+      </c>
+      <c r="B73" s="8" t="s">
+        <v>283</v>
+      </c>
+      <c r="C73" s="8">
         <v>1919</v>
       </c>
-      <c r="C73" s="9" t="s">
-        <v>211</v>
-      </c>
-      <c r="D73" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E73" s="9" t="s">
-        <v>214</v>
-      </c>
-      <c r="F73" s="10" t="s">
-        <v>215</v>
-      </c>
-      <c r="G73" s="10"/>
-    </row>
-    <row r="74" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="D73" s="9" t="s">
+        <v>281</v>
+      </c>
+      <c r="E73" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="F73" s="9" t="s">
+        <v>284</v>
+      </c>
+      <c r="G73" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="H73" s="10"/>
+    </row>
+    <row r="74" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A74" s="8">
         <v>69</v>
       </c>
       <c r="B74" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="C74" s="9" t="s">
-        <v>217</v>
-      </c>
-      <c r="D74" s="8"/>
-      <c r="E74" s="9" t="s">
-        <v>218</v>
-      </c>
-      <c r="F74" s="10" t="s">
-        <v>219</v>
+        <v>286</v>
+      </c>
+      <c r="C74" s="8" t="s">
+        <v>287</v>
+      </c>
+      <c r="D74" s="9" t="s">
+        <v>288</v>
+      </c>
+      <c r="E74" s="8"/>
+      <c r="F74" s="9" t="s">
+        <v>289</v>
       </c>
       <c r="G74" s="10" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="75" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>290</v>
+      </c>
+      <c r="H74" s="10" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="75" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A75" s="8">
         <v>70</v>
       </c>
-      <c r="B75" s="8">
+      <c r="B75" s="8" t="s">
+        <v>292</v>
+      </c>
+      <c r="C75" s="8">
         <v>1918</v>
       </c>
-      <c r="C75" s="9" t="s">
-        <v>221</v>
-      </c>
-      <c r="D75" s="8"/>
-      <c r="E75" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="F75" s="10" t="s">
-        <v>223</v>
+      <c r="D75" s="9" t="s">
+        <v>293</v>
+      </c>
+      <c r="E75" s="8"/>
+      <c r="F75" s="9" t="s">
+        <v>294</v>
       </c>
       <c r="G75" s="10" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="76" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>295</v>
+      </c>
+      <c r="H75" s="10" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="76" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A76" s="8">
         <v>71</v>
       </c>
       <c r="B76" s="8" t="s">
-        <v>225</v>
-      </c>
-      <c r="C76" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="D76" s="8"/>
-      <c r="E76" s="9"/>
-      <c r="F76" s="10" t="s">
-        <v>227</v>
-      </c>
+        <v>297</v>
+      </c>
+      <c r="C76" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="D76" s="9" t="s">
+        <v>299</v>
+      </c>
+      <c r="E76" s="8"/>
+      <c r="F76" s="9"/>
       <c r="G76" s="10" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="77" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>300</v>
+      </c>
+      <c r="H76" s="10" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="77" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A77" s="8">
         <v>72</v>
       </c>
       <c r="B77" s="8" t="s">
-        <v>229</v>
-      </c>
-      <c r="C77" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="D77" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="E77" s="9" t="s">
-        <v>231</v>
-      </c>
-      <c r="F77" s="10" t="s">
-        <v>232</v>
-      </c>
-      <c r="G77" s="10"/>
-    </row>
-    <row r="78" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>302</v>
+      </c>
+      <c r="C77" s="8" t="s">
+        <v>303</v>
+      </c>
+      <c r="D77" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="E77" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="F77" s="9" t="s">
+        <v>305</v>
+      </c>
+      <c r="G77" s="10" t="s">
+        <v>306</v>
+      </c>
+      <c r="H77" s="10"/>
+    </row>
+    <row r="78" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A78" s="8">
         <v>73</v>
       </c>
       <c r="B78" s="8" t="s">
-        <v>233</v>
-      </c>
-      <c r="C78" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="D78" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="E78" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="F78" s="10" t="s">
-        <v>235</v>
+        <v>307</v>
+      </c>
+      <c r="C78" s="8" t="s">
+        <v>308</v>
+      </c>
+      <c r="D78" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="E78" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="F78" s="9" t="s">
+        <v>309</v>
       </c>
       <c r="G78" s="10" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="79" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>310</v>
+      </c>
+      <c r="H78" s="10" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="79" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A79" s="8">
         <v>74</v>
       </c>
-      <c r="B79" s="8">
+      <c r="B79" s="8" t="s">
+        <v>312</v>
+      </c>
+      <c r="C79" s="8">
         <v>1922</v>
       </c>
-      <c r="C79" s="9" t="s">
-        <v>237</v>
-      </c>
-      <c r="D79" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="E79" s="9" t="s">
-        <v>238</v>
-      </c>
-      <c r="F79" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="G79" s="10"/>
-    </row>
-    <row r="80" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="D79" s="9" t="s">
+        <v>313</v>
+      </c>
+      <c r="E79" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="F79" s="9" t="s">
+        <v>314</v>
+      </c>
+      <c r="G79" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="H79" s="10"/>
+    </row>
+    <row r="80" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A80" s="8">
         <v>75</v>
       </c>
       <c r="B80" s="8" t="s">
-        <v>239</v>
-      </c>
-      <c r="C80" s="9" t="s">
-        <v>240</v>
-      </c>
-      <c r="D80" s="8"/>
-      <c r="E80" s="9"/>
-      <c r="F80" s="10" t="s">
-        <v>241</v>
-      </c>
+        <v>315</v>
+      </c>
+      <c r="C80" s="8" t="s">
+        <v>316</v>
+      </c>
+      <c r="D80" s="9" t="s">
+        <v>317</v>
+      </c>
+      <c r="E80" s="8"/>
+      <c r="F80" s="9"/>
       <c r="G80" s="10" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="81" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>318</v>
+      </c>
+      <c r="H80" s="10" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="81" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A81" s="8">
         <v>76</v>
       </c>
       <c r="B81" s="8" t="s">
-        <v>243</v>
-      </c>
-      <c r="C81" s="9" t="s">
-        <v>244</v>
-      </c>
-      <c r="D81" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="E81" s="9" t="s">
-        <v>245</v>
-      </c>
-      <c r="F81" s="10" t="s">
-        <v>246</v>
-      </c>
-      <c r="G81" s="10"/>
-    </row>
-    <row r="82" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>320</v>
+      </c>
+      <c r="C81" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="D81" s="9" t="s">
+        <v>322</v>
+      </c>
+      <c r="E81" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="F81" s="9" t="s">
+        <v>323</v>
+      </c>
+      <c r="G81" s="10" t="s">
+        <v>324</v>
+      </c>
+      <c r="H81" s="10"/>
+    </row>
+    <row r="82" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A82" s="8">
         <v>77</v>
       </c>
       <c r="B82" s="8" t="s">
-        <v>247</v>
-      </c>
-      <c r="C82" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="D82" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="E82" s="9" t="s">
-        <v>248</v>
-      </c>
-      <c r="F82" s="10" t="s">
-        <v>38</v>
+        <v>325</v>
+      </c>
+      <c r="C82" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="D82" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="E82" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="F82" s="9" t="s">
+        <v>327</v>
       </c>
       <c r="G82" s="10" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="83" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>49</v>
+      </c>
+      <c r="H82" s="10" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="83" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A83" s="8">
         <v>78</v>
       </c>
       <c r="B83" s="8" t="s">
-        <v>250</v>
-      </c>
-      <c r="C83" s="9" t="s">
-        <v>251</v>
-      </c>
-      <c r="D83" s="8"/>
-      <c r="E83" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="F83" s="10" t="s">
-        <v>253</v>
+        <v>329</v>
+      </c>
+      <c r="C83" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="D83" s="9" t="s">
+        <v>331</v>
+      </c>
+      <c r="E83" s="8"/>
+      <c r="F83" s="9" t="s">
+        <v>332</v>
       </c>
       <c r="G83" s="10" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="84" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>333</v>
+      </c>
+      <c r="H83" s="10" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="84" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A84" s="8">
         <v>79</v>
       </c>
-      <c r="B84" s="8">
+      <c r="B84" s="8" t="s">
+        <v>335</v>
+      </c>
+      <c r="C84" s="8">
         <v>1927</v>
       </c>
-      <c r="C84" s="9" t="s">
-        <v>255</v>
-      </c>
-      <c r="D84" s="8"/>
-      <c r="E84" s="9"/>
-      <c r="F84" s="10" t="s">
-        <v>17</v>
-      </c>
+      <c r="D84" s="9" t="s">
+        <v>336</v>
+      </c>
+      <c r="E84" s="8"/>
+      <c r="F84" s="9"/>
       <c r="G84" s="10" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="85" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>23</v>
+      </c>
+      <c r="H84" s="10" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="85" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A85" s="8">
         <v>80</v>
       </c>
-      <c r="B85" s="8">
+      <c r="B85" s="8" t="s">
+        <v>338</v>
+      </c>
+      <c r="C85" s="8">
         <v>1927</v>
       </c>
-      <c r="C85" s="9" t="s">
-        <v>257</v>
-      </c>
-      <c r="D85" s="8"/>
-      <c r="E85" s="9"/>
-      <c r="F85" s="10" t="s">
-        <v>258</v>
-      </c>
-      <c r="G85" s="10"/>
-    </row>
-    <row r="86" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="D85" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="E85" s="8"/>
+      <c r="F85" s="9"/>
+      <c r="G85" s="10" t="s">
+        <v>340</v>
+      </c>
+      <c r="H85" s="10"/>
+    </row>
+    <row r="86" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A86" s="8">
         <v>81</v>
       </c>
-      <c r="B86" s="8">
+      <c r="B86" s="8" t="s">
+        <v>341</v>
+      </c>
+      <c r="C86" s="8">
         <v>1928</v>
       </c>
-      <c r="C86" s="9" t="s">
-        <v>259</v>
-      </c>
-      <c r="D86" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="E86" s="9" t="s">
-        <v>260</v>
-      </c>
-      <c r="F86" s="10" t="s">
-        <v>261</v>
+      <c r="D86" s="9" t="s">
+        <v>342</v>
+      </c>
+      <c r="E86" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="F86" s="9" t="s">
+        <v>343</v>
       </c>
       <c r="G86" s="10" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="87" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>344</v>
+      </c>
+      <c r="H86" s="10" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="87" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A87" s="8">
         <v>82</v>
       </c>
       <c r="B87" s="8" t="s">
-        <v>263</v>
-      </c>
-      <c r="C87" s="9" t="s">
-        <v>264</v>
-      </c>
-      <c r="D87" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="E87" s="9" t="s">
-        <v>265</v>
-      </c>
-      <c r="F87" s="10" t="s">
-        <v>266</v>
+        <v>346</v>
+      </c>
+      <c r="C87" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="D87" s="9" t="s">
+        <v>348</v>
+      </c>
+      <c r="E87" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="F87" s="9" t="s">
+        <v>349</v>
       </c>
       <c r="G87" s="10" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="88" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>350</v>
+      </c>
+      <c r="H87" s="10" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="88" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A88" s="8">
         <v>83</v>
       </c>
       <c r="B88" s="8" t="s">
-        <v>268</v>
-      </c>
-      <c r="C88" s="9" t="s">
-        <v>264</v>
-      </c>
-      <c r="D88" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="E88" s="9" t="s">
-        <v>269</v>
-      </c>
-      <c r="F88" s="10" t="s">
-        <v>270</v>
+        <v>352</v>
+      </c>
+      <c r="C88" s="8" t="s">
+        <v>353</v>
+      </c>
+      <c r="D88" s="9" t="s">
+        <v>348</v>
+      </c>
+      <c r="E88" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="F88" s="9" t="s">
+        <v>354</v>
       </c>
       <c r="G88" s="10" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="89" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>355</v>
+      </c>
+      <c r="H88" s="10" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="89" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A89" s="8">
         <v>84</v>
       </c>
       <c r="B89" s="8" t="s">
-        <v>272</v>
-      </c>
-      <c r="C89" s="9" t="s">
-        <v>273</v>
-      </c>
-      <c r="D89" s="8"/>
-      <c r="E89" s="9" t="s">
-        <v>274</v>
-      </c>
-      <c r="F89" s="10" t="s">
-        <v>275</v>
+        <v>357</v>
+      </c>
+      <c r="C89" s="8" t="s">
+        <v>358</v>
+      </c>
+      <c r="D89" s="9" t="s">
+        <v>359</v>
+      </c>
+      <c r="E89" s="8"/>
+      <c r="F89" s="9" t="s">
+        <v>360</v>
       </c>
       <c r="G89" s="10" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="90" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>361</v>
+      </c>
+      <c r="H89" s="10" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="90" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A90" s="8">
         <v>85</v>
       </c>
-      <c r="B90" s="8">
+      <c r="B90" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="C90" s="8">
         <v>1932</v>
       </c>
-      <c r="C90" s="9" t="s">
-        <v>277</v>
-      </c>
-      <c r="D90" s="8"/>
-      <c r="E90" s="9"/>
-      <c r="F90" s="10" t="s">
-        <v>278</v>
-      </c>
+      <c r="D90" s="9" t="s">
+        <v>364</v>
+      </c>
+      <c r="E90" s="8"/>
+      <c r="F90" s="9"/>
       <c r="G90" s="10" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="91" s="2" customFormat="1" customHeight="1" spans="1:7">
+        <v>365</v>
+      </c>
+      <c r="H90" s="10" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="91" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A91" s="3"/>
       <c r="B91" s="3"/>
-      <c r="C91" s="4"/>
-      <c r="D91" s="3"/>
-      <c r="E91" s="5"/>
+      <c r="C91" s="3"/>
+      <c r="D91" s="4"/>
+      <c r="E91" s="3"/>
       <c r="F91" s="5"/>
       <c r="G91" s="5"/>
-    </row>
-    <row r="92" s="2" customFormat="1" customHeight="1" spans="1:7">
+      <c r="H91" s="5"/>
+    </row>
+    <row r="92" s="2" customFormat="1" customHeight="1" spans="1:8">
       <c r="A92" s="3"/>
       <c r="B92" s="3"/>
-      <c r="C92" s="4"/>
-      <c r="D92" s="3"/>
-      <c r="E92" s="5"/>
+      <c r="C92" s="3"/>
+      <c r="D92" s="4"/>
+      <c r="E92" s="3"/>
       <c r="F92" s="5"/>
       <c r="G92" s="5"/>
+      <c r="H92" s="5"/>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:G92" etc:filterBottomFollowUsedRange="0">
-    <sortState ref="A1:G92">
-      <sortCondition ref="A1"/>
-    </sortState>
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H92" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>